<commit_message>
docs(validation): R8.1 checklist items for throttling, secret permissions, report descriptions and test tooling
Adds R81-01 to R81-15 (all Not tested, approval Pending; the Windows, Docker and
systemd items are Partially implemented with the reason), supersedes the wording
of R8-01 and SEC-003 with their earlier text kept in Notes, and regenerates the
workbook. No reviewer status, date or approval was changed.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EsCXzFEofbBScBiLBFpRK2
</commit_message>
<xml_diff>
--- a/docs/validation/validation-tracker.xlsx
+++ b/docs/validation/validation-tracker.xlsx
@@ -133,8 +133,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ValidationItems" displayName="ValidationItems" ref="A1:S196" totalsRowShown="0">
-  <autoFilter ref="A1:S196"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ValidationItems" displayName="ValidationItems" ref="A1:S211" totalsRowShown="0">
+  <autoFilter ref="A1:S211"/>
   <tableColumns count="19">
     <tableColumn id="1" name="ID"/>
     <tableColumn id="2" name="Area"/>
@@ -267,39 +267,39 @@
         </is>
       </c>
       <c r="B6" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$196,$A6)</f>
+        <f>COUNTIFS(Items!$B$2:$B$211,$A6)</f>
         <v>9</v>
       </c>
       <c r="C6" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$196,$A6,Items!$F$2:$F$196,C$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$211,$A6,Items!$F$2:$F$211,C$5)</f>
         <v>9</v>
       </c>
       <c r="D6" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$196,$A6,Items!$F$2:$F$196,D$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$211,$A6,Items!$F$2:$F$211,D$5)</f>
         <v>0</v>
       </c>
       <c r="E6" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$196,$A6,Items!$F$2:$F$196,E$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$211,$A6,Items!$F$2:$F$211,E$5)</f>
         <v>0</v>
       </c>
       <c r="F6" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$196,$A6,Items!$F$2:$F$196,F$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$211,$A6,Items!$F$2:$F$211,F$5)</f>
         <v>0</v>
       </c>
       <c r="G6" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$196,$A6,Items!$F$2:$F$196,G$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$211,$A6,Items!$F$2:$F$211,G$5)</f>
         <v>0</v>
       </c>
       <c r="H6" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$196,$A6,Items!$F$2:$F$196,H$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$211,$A6,Items!$F$2:$F$211,H$5)</f>
         <v>0</v>
       </c>
       <c r="I6" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$196,$A6,Items!$G$2:$G$196,"Approved")</f>
+        <f>COUNTIFS(Items!$B$2:$B$211,$A6,Items!$G$2:$G$211,"Approved")</f>
         <v>0</v>
       </c>
       <c r="J6" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$196,$A6,Items!$G$2:$G$196,"Pending")</f>
+        <f>COUNTIFS(Items!$B$2:$B$211,$A6,Items!$G$2:$G$211,"Pending")</f>
         <v>9</v>
       </c>
       <c r="K6" s="4">
@@ -318,40 +318,40 @@
         </is>
       </c>
       <c r="B7" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$196,$A7)</f>
-        <v>9</v>
+        <f>COUNTIFS(Items!$B$2:$B$211,$A7)</f>
+        <v>10</v>
       </c>
       <c r="C7" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$196,$A7,Items!$F$2:$F$196,C$5)</f>
-        <v>9</v>
+        <f>COUNTIFS(Items!$B$2:$B$211,$A7,Items!$F$2:$F$211,C$5)</f>
+        <v>10</v>
       </c>
       <c r="D7" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$196,$A7,Items!$F$2:$F$196,D$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$211,$A7,Items!$F$2:$F$211,D$5)</f>
         <v>0</v>
       </c>
       <c r="E7" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$196,$A7,Items!$F$2:$F$196,E$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$211,$A7,Items!$F$2:$F$211,E$5)</f>
         <v>0</v>
       </c>
       <c r="F7" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$196,$A7,Items!$F$2:$F$196,F$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$211,$A7,Items!$F$2:$F$211,F$5)</f>
         <v>0</v>
       </c>
       <c r="G7" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$196,$A7,Items!$F$2:$F$196,G$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$211,$A7,Items!$F$2:$F$211,G$5)</f>
         <v>0</v>
       </c>
       <c r="H7" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$196,$A7,Items!$F$2:$F$196,H$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$211,$A7,Items!$F$2:$F$211,H$5)</f>
         <v>0</v>
       </c>
       <c r="I7" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$196,$A7,Items!$G$2:$G$196,"Approved")</f>
+        <f>COUNTIFS(Items!$B$2:$B$211,$A7,Items!$G$2:$G$211,"Approved")</f>
         <v>0</v>
       </c>
       <c r="J7" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$196,$A7,Items!$G$2:$G$196,"Pending")</f>
-        <v>9</v>
+        <f>COUNTIFS(Items!$B$2:$B$211,$A7,Items!$G$2:$G$211,"Pending")</f>
+        <v>10</v>
       </c>
       <c r="K7" s="4">
         <f>IF(B7-G7=0,0,(D7+E7+F7)/(B7-G7))</f>
@@ -369,39 +369,39 @@
         </is>
       </c>
       <c r="B8" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$196,$A8)</f>
+        <f>COUNTIFS(Items!$B$2:$B$211,$A8)</f>
         <v>9</v>
       </c>
       <c r="C8" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$196,$A8,Items!$F$2:$F$196,C$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$211,$A8,Items!$F$2:$F$211,C$5)</f>
         <v>8</v>
       </c>
       <c r="D8" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$196,$A8,Items!$F$2:$F$196,D$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$211,$A8,Items!$F$2:$F$211,D$5)</f>
         <v>0</v>
       </c>
       <c r="E8" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$196,$A8,Items!$F$2:$F$196,E$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$211,$A8,Items!$F$2:$F$211,E$5)</f>
         <v>0</v>
       </c>
       <c r="F8" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$196,$A8,Items!$F$2:$F$196,F$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$211,$A8,Items!$F$2:$F$211,F$5)</f>
         <v>1</v>
       </c>
       <c r="G8" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$196,$A8,Items!$F$2:$F$196,G$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$211,$A8,Items!$F$2:$F$211,G$5)</f>
         <v>0</v>
       </c>
       <c r="H8" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$196,$A8,Items!$F$2:$F$196,H$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$211,$A8,Items!$F$2:$F$211,H$5)</f>
         <v>0</v>
       </c>
       <c r="I8" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$196,$A8,Items!$G$2:$G$196,"Approved")</f>
+        <f>COUNTIFS(Items!$B$2:$B$211,$A8,Items!$G$2:$G$211,"Approved")</f>
         <v>0</v>
       </c>
       <c r="J8" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$196,$A8,Items!$G$2:$G$196,"Pending")</f>
+        <f>COUNTIFS(Items!$B$2:$B$211,$A8,Items!$G$2:$G$211,"Pending")</f>
         <v>9</v>
       </c>
       <c r="K8" s="4">
@@ -420,39 +420,39 @@
         </is>
       </c>
       <c r="B9" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$196,$A9)</f>
+        <f>COUNTIFS(Items!$B$2:$B$211,$A9)</f>
         <v>9</v>
       </c>
       <c r="C9" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$196,$A9,Items!$F$2:$F$196,C$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$211,$A9,Items!$F$2:$F$211,C$5)</f>
         <v>9</v>
       </c>
       <c r="D9" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$196,$A9,Items!$F$2:$F$196,D$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$211,$A9,Items!$F$2:$F$211,D$5)</f>
         <v>0</v>
       </c>
       <c r="E9" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$196,$A9,Items!$F$2:$F$196,E$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$211,$A9,Items!$F$2:$F$211,E$5)</f>
         <v>0</v>
       </c>
       <c r="F9" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$196,$A9,Items!$F$2:$F$196,F$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$211,$A9,Items!$F$2:$F$211,F$5)</f>
         <v>0</v>
       </c>
       <c r="G9" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$196,$A9,Items!$F$2:$F$196,G$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$211,$A9,Items!$F$2:$F$211,G$5)</f>
         <v>0</v>
       </c>
       <c r="H9" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$196,$A9,Items!$F$2:$F$196,H$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$211,$A9,Items!$F$2:$F$211,H$5)</f>
         <v>0</v>
       </c>
       <c r="I9" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$196,$A9,Items!$G$2:$G$196,"Approved")</f>
+        <f>COUNTIFS(Items!$B$2:$B$211,$A9,Items!$G$2:$G$211,"Approved")</f>
         <v>0</v>
       </c>
       <c r="J9" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$196,$A9,Items!$G$2:$G$196,"Pending")</f>
+        <f>COUNTIFS(Items!$B$2:$B$211,$A9,Items!$G$2:$G$211,"Pending")</f>
         <v>9</v>
       </c>
       <c r="K9" s="4">
@@ -471,39 +471,39 @@
         </is>
       </c>
       <c r="B10" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$196,$A10)</f>
+        <f>COUNTIFS(Items!$B$2:$B$211,$A10)</f>
         <v>9</v>
       </c>
       <c r="C10" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$196,$A10,Items!$F$2:$F$196,C$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$211,$A10,Items!$F$2:$F$211,C$5)</f>
         <v>9</v>
       </c>
       <c r="D10" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$196,$A10,Items!$F$2:$F$196,D$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$211,$A10,Items!$F$2:$F$211,D$5)</f>
         <v>0</v>
       </c>
       <c r="E10" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$196,$A10,Items!$F$2:$F$196,E$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$211,$A10,Items!$F$2:$F$211,E$5)</f>
         <v>0</v>
       </c>
       <c r="F10" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$196,$A10,Items!$F$2:$F$196,F$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$211,$A10,Items!$F$2:$F$211,F$5)</f>
         <v>0</v>
       </c>
       <c r="G10" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$196,$A10,Items!$F$2:$F$196,G$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$211,$A10,Items!$F$2:$F$211,G$5)</f>
         <v>0</v>
       </c>
       <c r="H10" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$196,$A10,Items!$F$2:$F$196,H$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$211,$A10,Items!$F$2:$F$211,H$5)</f>
         <v>0</v>
       </c>
       <c r="I10" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$196,$A10,Items!$G$2:$G$196,"Approved")</f>
+        <f>COUNTIFS(Items!$B$2:$B$211,$A10,Items!$G$2:$G$211,"Approved")</f>
         <v>0</v>
       </c>
       <c r="J10" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$196,$A10,Items!$G$2:$G$196,"Pending")</f>
+        <f>COUNTIFS(Items!$B$2:$B$211,$A10,Items!$G$2:$G$211,"Pending")</f>
         <v>9</v>
       </c>
       <c r="K10" s="4">
@@ -522,39 +522,39 @@
         </is>
       </c>
       <c r="B11" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$196,$A11)</f>
+        <f>COUNTIFS(Items!$B$2:$B$211,$A11)</f>
         <v>5</v>
       </c>
       <c r="C11" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$196,$A11,Items!$F$2:$F$196,C$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$211,$A11,Items!$F$2:$F$211,C$5)</f>
         <v>5</v>
       </c>
       <c r="D11" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$196,$A11,Items!$F$2:$F$196,D$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$211,$A11,Items!$F$2:$F$211,D$5)</f>
         <v>0</v>
       </c>
       <c r="E11" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$196,$A11,Items!$F$2:$F$196,E$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$211,$A11,Items!$F$2:$F$211,E$5)</f>
         <v>0</v>
       </c>
       <c r="F11" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$196,$A11,Items!$F$2:$F$196,F$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$211,$A11,Items!$F$2:$F$211,F$5)</f>
         <v>0</v>
       </c>
       <c r="G11" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$196,$A11,Items!$F$2:$F$196,G$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$211,$A11,Items!$F$2:$F$211,G$5)</f>
         <v>0</v>
       </c>
       <c r="H11" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$196,$A11,Items!$F$2:$F$196,H$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$211,$A11,Items!$F$2:$F$211,H$5)</f>
         <v>0</v>
       </c>
       <c r="I11" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$196,$A11,Items!$G$2:$G$196,"Approved")</f>
+        <f>COUNTIFS(Items!$B$2:$B$211,$A11,Items!$G$2:$G$211,"Approved")</f>
         <v>0</v>
       </c>
       <c r="J11" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$196,$A11,Items!$G$2:$G$196,"Pending")</f>
+        <f>COUNTIFS(Items!$B$2:$B$211,$A11,Items!$G$2:$G$211,"Pending")</f>
         <v>5</v>
       </c>
       <c r="K11" s="4">
@@ -573,39 +573,39 @@
         </is>
       </c>
       <c r="B12" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$196,$A12)</f>
+        <f>COUNTIFS(Items!$B$2:$B$211,$A12)</f>
         <v>5</v>
       </c>
       <c r="C12" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$196,$A12,Items!$F$2:$F$196,C$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$211,$A12,Items!$F$2:$F$211,C$5)</f>
         <v>5</v>
       </c>
       <c r="D12" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$196,$A12,Items!$F$2:$F$196,D$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$211,$A12,Items!$F$2:$F$211,D$5)</f>
         <v>0</v>
       </c>
       <c r="E12" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$196,$A12,Items!$F$2:$F$196,E$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$211,$A12,Items!$F$2:$F$211,E$5)</f>
         <v>0</v>
       </c>
       <c r="F12" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$196,$A12,Items!$F$2:$F$196,F$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$211,$A12,Items!$F$2:$F$211,F$5)</f>
         <v>0</v>
       </c>
       <c r="G12" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$196,$A12,Items!$F$2:$F$196,G$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$211,$A12,Items!$F$2:$F$211,G$5)</f>
         <v>0</v>
       </c>
       <c r="H12" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$196,$A12,Items!$F$2:$F$196,H$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$211,$A12,Items!$F$2:$F$211,H$5)</f>
         <v>0</v>
       </c>
       <c r="I12" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$196,$A12,Items!$G$2:$G$196,"Approved")</f>
+        <f>COUNTIFS(Items!$B$2:$B$211,$A12,Items!$G$2:$G$211,"Approved")</f>
         <v>0</v>
       </c>
       <c r="J12" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$196,$A12,Items!$G$2:$G$196,"Pending")</f>
+        <f>COUNTIFS(Items!$B$2:$B$211,$A12,Items!$G$2:$G$211,"Pending")</f>
         <v>5</v>
       </c>
       <c r="K12" s="4">
@@ -624,39 +624,39 @@
         </is>
       </c>
       <c r="B13" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$196,$A13)</f>
+        <f>COUNTIFS(Items!$B$2:$B$211,$A13)</f>
         <v>9</v>
       </c>
       <c r="C13" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$196,$A13,Items!$F$2:$F$196,C$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$211,$A13,Items!$F$2:$F$211,C$5)</f>
         <v>9</v>
       </c>
       <c r="D13" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$196,$A13,Items!$F$2:$F$196,D$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$211,$A13,Items!$F$2:$F$211,D$5)</f>
         <v>0</v>
       </c>
       <c r="E13" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$196,$A13,Items!$F$2:$F$196,E$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$211,$A13,Items!$F$2:$F$211,E$5)</f>
         <v>0</v>
       </c>
       <c r="F13" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$196,$A13,Items!$F$2:$F$196,F$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$211,$A13,Items!$F$2:$F$211,F$5)</f>
         <v>0</v>
       </c>
       <c r="G13" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$196,$A13,Items!$F$2:$F$196,G$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$211,$A13,Items!$F$2:$F$211,G$5)</f>
         <v>0</v>
       </c>
       <c r="H13" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$196,$A13,Items!$F$2:$F$196,H$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$211,$A13,Items!$F$2:$F$211,H$5)</f>
         <v>0</v>
       </c>
       <c r="I13" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$196,$A13,Items!$G$2:$G$196,"Approved")</f>
+        <f>COUNTIFS(Items!$B$2:$B$211,$A13,Items!$G$2:$G$211,"Approved")</f>
         <v>0</v>
       </c>
       <c r="J13" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$196,$A13,Items!$G$2:$G$196,"Pending")</f>
+        <f>COUNTIFS(Items!$B$2:$B$211,$A13,Items!$G$2:$G$211,"Pending")</f>
         <v>9</v>
       </c>
       <c r="K13" s="4">
@@ -675,39 +675,39 @@
         </is>
       </c>
       <c r="B14" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$196,$A14)</f>
+        <f>COUNTIFS(Items!$B$2:$B$211,$A14)</f>
         <v>17</v>
       </c>
       <c r="C14" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$196,$A14,Items!$F$2:$F$196,C$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$211,$A14,Items!$F$2:$F$211,C$5)</f>
         <v>17</v>
       </c>
       <c r="D14" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$196,$A14,Items!$F$2:$F$196,D$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$211,$A14,Items!$F$2:$F$211,D$5)</f>
         <v>0</v>
       </c>
       <c r="E14" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$196,$A14,Items!$F$2:$F$196,E$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$211,$A14,Items!$F$2:$F$211,E$5)</f>
         <v>0</v>
       </c>
       <c r="F14" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$196,$A14,Items!$F$2:$F$196,F$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$211,$A14,Items!$F$2:$F$211,F$5)</f>
         <v>0</v>
       </c>
       <c r="G14" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$196,$A14,Items!$F$2:$F$196,G$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$211,$A14,Items!$F$2:$F$211,G$5)</f>
         <v>0</v>
       </c>
       <c r="H14" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$196,$A14,Items!$F$2:$F$196,H$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$211,$A14,Items!$F$2:$F$211,H$5)</f>
         <v>0</v>
       </c>
       <c r="I14" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$196,$A14,Items!$G$2:$G$196,"Approved")</f>
+        <f>COUNTIFS(Items!$B$2:$B$211,$A14,Items!$G$2:$G$211,"Approved")</f>
         <v>0</v>
       </c>
       <c r="J14" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$196,$A14,Items!$G$2:$G$196,"Pending")</f>
+        <f>COUNTIFS(Items!$B$2:$B$211,$A14,Items!$G$2:$G$211,"Pending")</f>
         <v>17</v>
       </c>
       <c r="K14" s="4">
@@ -726,39 +726,39 @@
         </is>
       </c>
       <c r="B15" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$196,$A15)</f>
+        <f>COUNTIFS(Items!$B$2:$B$211,$A15)</f>
         <v>4</v>
       </c>
       <c r="C15" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$196,$A15,Items!$F$2:$F$196,C$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$211,$A15,Items!$F$2:$F$211,C$5)</f>
         <v>4</v>
       </c>
       <c r="D15" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$196,$A15,Items!$F$2:$F$196,D$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$211,$A15,Items!$F$2:$F$211,D$5)</f>
         <v>0</v>
       </c>
       <c r="E15" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$196,$A15,Items!$F$2:$F$196,E$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$211,$A15,Items!$F$2:$F$211,E$5)</f>
         <v>0</v>
       </c>
       <c r="F15" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$196,$A15,Items!$F$2:$F$196,F$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$211,$A15,Items!$F$2:$F$211,F$5)</f>
         <v>0</v>
       </c>
       <c r="G15" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$196,$A15,Items!$F$2:$F$196,G$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$211,$A15,Items!$F$2:$F$211,G$5)</f>
         <v>0</v>
       </c>
       <c r="H15" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$196,$A15,Items!$F$2:$F$196,H$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$211,$A15,Items!$F$2:$F$211,H$5)</f>
         <v>0</v>
       </c>
       <c r="I15" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$196,$A15,Items!$G$2:$G$196,"Approved")</f>
+        <f>COUNTIFS(Items!$B$2:$B$211,$A15,Items!$G$2:$G$211,"Approved")</f>
         <v>0</v>
       </c>
       <c r="J15" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$196,$A15,Items!$G$2:$G$196,"Pending")</f>
+        <f>COUNTIFS(Items!$B$2:$B$211,$A15,Items!$G$2:$G$211,"Pending")</f>
         <v>4</v>
       </c>
       <c r="K15" s="4">
@@ -777,39 +777,39 @@
         </is>
       </c>
       <c r="B16" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$196,$A16)</f>
+        <f>COUNTIFS(Items!$B$2:$B$211,$A16)</f>
         <v>9</v>
       </c>
       <c r="C16" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$196,$A16,Items!$F$2:$F$196,C$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$211,$A16,Items!$F$2:$F$211,C$5)</f>
         <v>9</v>
       </c>
       <c r="D16" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$196,$A16,Items!$F$2:$F$196,D$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$211,$A16,Items!$F$2:$F$211,D$5)</f>
         <v>0</v>
       </c>
       <c r="E16" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$196,$A16,Items!$F$2:$F$196,E$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$211,$A16,Items!$F$2:$F$211,E$5)</f>
         <v>0</v>
       </c>
       <c r="F16" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$196,$A16,Items!$F$2:$F$196,F$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$211,$A16,Items!$F$2:$F$211,F$5)</f>
         <v>0</v>
       </c>
       <c r="G16" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$196,$A16,Items!$F$2:$F$196,G$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$211,$A16,Items!$F$2:$F$211,G$5)</f>
         <v>0</v>
       </c>
       <c r="H16" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$196,$A16,Items!$F$2:$F$196,H$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$211,$A16,Items!$F$2:$F$211,H$5)</f>
         <v>0</v>
       </c>
       <c r="I16" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$196,$A16,Items!$G$2:$G$196,"Approved")</f>
+        <f>COUNTIFS(Items!$B$2:$B$211,$A16,Items!$G$2:$G$211,"Approved")</f>
         <v>0</v>
       </c>
       <c r="J16" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$196,$A16,Items!$G$2:$G$196,"Pending")</f>
+        <f>COUNTIFS(Items!$B$2:$B$211,$A16,Items!$G$2:$G$211,"Pending")</f>
         <v>9</v>
       </c>
       <c r="K16" s="4">
@@ -828,39 +828,39 @@
         </is>
       </c>
       <c r="B17" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$196,$A17)</f>
+        <f>COUNTIFS(Items!$B$2:$B$211,$A17)</f>
         <v>15</v>
       </c>
       <c r="C17" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$196,$A17,Items!$F$2:$F$196,C$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$211,$A17,Items!$F$2:$F$211,C$5)</f>
         <v>14</v>
       </c>
       <c r="D17" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$196,$A17,Items!$F$2:$F$196,D$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$211,$A17,Items!$F$2:$F$211,D$5)</f>
         <v>0</v>
       </c>
       <c r="E17" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$196,$A17,Items!$F$2:$F$196,E$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$211,$A17,Items!$F$2:$F$211,E$5)</f>
         <v>0</v>
       </c>
       <c r="F17" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$196,$A17,Items!$F$2:$F$196,F$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$211,$A17,Items!$F$2:$F$211,F$5)</f>
         <v>1</v>
       </c>
       <c r="G17" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$196,$A17,Items!$F$2:$F$196,G$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$211,$A17,Items!$F$2:$F$211,G$5)</f>
         <v>0</v>
       </c>
       <c r="H17" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$196,$A17,Items!$F$2:$F$196,H$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$211,$A17,Items!$F$2:$F$211,H$5)</f>
         <v>0</v>
       </c>
       <c r="I17" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$196,$A17,Items!$G$2:$G$196,"Approved")</f>
+        <f>COUNTIFS(Items!$B$2:$B$211,$A17,Items!$G$2:$G$211,"Approved")</f>
         <v>0</v>
       </c>
       <c r="J17" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$196,$A17,Items!$G$2:$G$196,"Pending")</f>
+        <f>COUNTIFS(Items!$B$2:$B$211,$A17,Items!$G$2:$G$211,"Pending")</f>
         <v>15</v>
       </c>
       <c r="K17" s="4">
@@ -879,40 +879,40 @@
         </is>
       </c>
       <c r="B18" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$196,$A18)</f>
-        <v>9</v>
+        <f>COUNTIFS(Items!$B$2:$B$211,$A18)</f>
+        <v>10</v>
       </c>
       <c r="C18" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$196,$A18,Items!$F$2:$F$196,C$5)</f>
-        <v>9</v>
+        <f>COUNTIFS(Items!$B$2:$B$211,$A18,Items!$F$2:$F$211,C$5)</f>
+        <v>10</v>
       </c>
       <c r="D18" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$196,$A18,Items!$F$2:$F$196,D$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$211,$A18,Items!$F$2:$F$211,D$5)</f>
         <v>0</v>
       </c>
       <c r="E18" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$196,$A18,Items!$F$2:$F$196,E$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$211,$A18,Items!$F$2:$F$211,E$5)</f>
         <v>0</v>
       </c>
       <c r="F18" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$196,$A18,Items!$F$2:$F$196,F$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$211,$A18,Items!$F$2:$F$211,F$5)</f>
         <v>0</v>
       </c>
       <c r="G18" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$196,$A18,Items!$F$2:$F$196,G$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$211,$A18,Items!$F$2:$F$211,G$5)</f>
         <v>0</v>
       </c>
       <c r="H18" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$196,$A18,Items!$F$2:$F$196,H$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$211,$A18,Items!$F$2:$F$211,H$5)</f>
         <v>0</v>
       </c>
       <c r="I18" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$196,$A18,Items!$G$2:$G$196,"Approved")</f>
+        <f>COUNTIFS(Items!$B$2:$B$211,$A18,Items!$G$2:$G$211,"Approved")</f>
         <v>0</v>
       </c>
       <c r="J18" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$196,$A18,Items!$G$2:$G$196,"Pending")</f>
-        <v>9</v>
+        <f>COUNTIFS(Items!$B$2:$B$211,$A18,Items!$G$2:$G$211,"Pending")</f>
+        <v>10</v>
       </c>
       <c r="K18" s="4">
         <f>IF(B18-G18=0,0,(D18+E18+F18)/(B18-G18))</f>
@@ -930,40 +930,40 @@
         </is>
       </c>
       <c r="B19" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$196,$A19)</f>
-        <v>4</v>
+        <f>COUNTIFS(Items!$B$2:$B$211,$A19)</f>
+        <v>7</v>
       </c>
       <c r="C19" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$196,$A19,Items!$F$2:$F$196,C$5)</f>
-        <v>4</v>
+        <f>COUNTIFS(Items!$B$2:$B$211,$A19,Items!$F$2:$F$211,C$5)</f>
+        <v>7</v>
       </c>
       <c r="D19" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$196,$A19,Items!$F$2:$F$196,D$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$211,$A19,Items!$F$2:$F$211,D$5)</f>
         <v>0</v>
       </c>
       <c r="E19" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$196,$A19,Items!$F$2:$F$196,E$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$211,$A19,Items!$F$2:$F$211,E$5)</f>
         <v>0</v>
       </c>
       <c r="F19" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$196,$A19,Items!$F$2:$F$196,F$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$211,$A19,Items!$F$2:$F$211,F$5)</f>
         <v>0</v>
       </c>
       <c r="G19" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$196,$A19,Items!$F$2:$F$196,G$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$211,$A19,Items!$F$2:$F$211,G$5)</f>
         <v>0</v>
       </c>
       <c r="H19" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$196,$A19,Items!$F$2:$F$196,H$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$211,$A19,Items!$F$2:$F$211,H$5)</f>
         <v>0</v>
       </c>
       <c r="I19" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$196,$A19,Items!$G$2:$G$196,"Approved")</f>
+        <f>COUNTIFS(Items!$B$2:$B$211,$A19,Items!$G$2:$G$211,"Approved")</f>
         <v>0</v>
       </c>
       <c r="J19" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$196,$A19,Items!$G$2:$G$196,"Pending")</f>
-        <v>4</v>
+        <f>COUNTIFS(Items!$B$2:$B$211,$A19,Items!$G$2:$G$211,"Pending")</f>
+        <v>7</v>
       </c>
       <c r="K19" s="4">
         <f>IF(B19-G19=0,0,(D19+E19+F19)/(B19-G19))</f>
@@ -981,40 +981,40 @@
         </is>
       </c>
       <c r="B20" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$196,$A20)</f>
-        <v>22</v>
+        <f>COUNTIFS(Items!$B$2:$B$211,$A20)</f>
+        <v>23</v>
       </c>
       <c r="C20" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$196,$A20,Items!$F$2:$F$196,C$5)</f>
-        <v>22</v>
+        <f>COUNTIFS(Items!$B$2:$B$211,$A20,Items!$F$2:$F$211,C$5)</f>
+        <v>23</v>
       </c>
       <c r="D20" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$196,$A20,Items!$F$2:$F$196,D$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$211,$A20,Items!$F$2:$F$211,D$5)</f>
         <v>0</v>
       </c>
       <c r="E20" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$196,$A20,Items!$F$2:$F$196,E$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$211,$A20,Items!$F$2:$F$211,E$5)</f>
         <v>0</v>
       </c>
       <c r="F20" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$196,$A20,Items!$F$2:$F$196,F$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$211,$A20,Items!$F$2:$F$211,F$5)</f>
         <v>0</v>
       </c>
       <c r="G20" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$196,$A20,Items!$F$2:$F$196,G$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$211,$A20,Items!$F$2:$F$211,G$5)</f>
         <v>0</v>
       </c>
       <c r="H20" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$196,$A20,Items!$F$2:$F$196,H$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$211,$A20,Items!$F$2:$F$211,H$5)</f>
         <v>0</v>
       </c>
       <c r="I20" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$196,$A20,Items!$G$2:$G$196,"Approved")</f>
+        <f>COUNTIFS(Items!$B$2:$B$211,$A20,Items!$G$2:$G$211,"Approved")</f>
         <v>0</v>
       </c>
       <c r="J20" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$196,$A20,Items!$G$2:$G$196,"Pending")</f>
-        <v>22</v>
+        <f>COUNTIFS(Items!$B$2:$B$211,$A20,Items!$G$2:$G$211,"Pending")</f>
+        <v>23</v>
       </c>
       <c r="K20" s="4">
         <f>IF(B20-G20=0,0,(D20+E20+F20)/(B20-G20))</f>
@@ -1032,39 +1032,39 @@
         </is>
       </c>
       <c r="B21" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$196,$A21)</f>
+        <f>COUNTIFS(Items!$B$2:$B$211,$A21)</f>
         <v>2</v>
       </c>
       <c r="C21" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$196,$A21,Items!$F$2:$F$196,C$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$211,$A21,Items!$F$2:$F$211,C$5)</f>
         <v>2</v>
       </c>
       <c r="D21" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$196,$A21,Items!$F$2:$F$196,D$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$211,$A21,Items!$F$2:$F$211,D$5)</f>
         <v>0</v>
       </c>
       <c r="E21" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$196,$A21,Items!$F$2:$F$196,E$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$211,$A21,Items!$F$2:$F$211,E$5)</f>
         <v>0</v>
       </c>
       <c r="F21" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$196,$A21,Items!$F$2:$F$196,F$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$211,$A21,Items!$F$2:$F$211,F$5)</f>
         <v>0</v>
       </c>
       <c r="G21" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$196,$A21,Items!$F$2:$F$196,G$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$211,$A21,Items!$F$2:$F$211,G$5)</f>
         <v>0</v>
       </c>
       <c r="H21" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$196,$A21,Items!$F$2:$F$196,H$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$211,$A21,Items!$F$2:$F$211,H$5)</f>
         <v>0</v>
       </c>
       <c r="I21" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$196,$A21,Items!$G$2:$G$196,"Approved")</f>
+        <f>COUNTIFS(Items!$B$2:$B$211,$A21,Items!$G$2:$G$211,"Approved")</f>
         <v>0</v>
       </c>
       <c r="J21" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$196,$A21,Items!$G$2:$G$196,"Pending")</f>
+        <f>COUNTIFS(Items!$B$2:$B$211,$A21,Items!$G$2:$G$211,"Pending")</f>
         <v>2</v>
       </c>
       <c r="K21" s="4">
@@ -1083,39 +1083,39 @@
         </is>
       </c>
       <c r="B22" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$196,$A22)</f>
+        <f>COUNTIFS(Items!$B$2:$B$211,$A22)</f>
         <v>6</v>
       </c>
       <c r="C22" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$196,$A22,Items!$F$2:$F$196,C$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$211,$A22,Items!$F$2:$F$211,C$5)</f>
         <v>6</v>
       </c>
       <c r="D22" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$196,$A22,Items!$F$2:$F$196,D$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$211,$A22,Items!$F$2:$F$211,D$5)</f>
         <v>0</v>
       </c>
       <c r="E22" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$196,$A22,Items!$F$2:$F$196,E$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$211,$A22,Items!$F$2:$F$211,E$5)</f>
         <v>0</v>
       </c>
       <c r="F22" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$196,$A22,Items!$F$2:$F$196,F$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$211,$A22,Items!$F$2:$F$211,F$5)</f>
         <v>0</v>
       </c>
       <c r="G22" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$196,$A22,Items!$F$2:$F$196,G$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$211,$A22,Items!$F$2:$F$211,G$5)</f>
         <v>0</v>
       </c>
       <c r="H22" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$196,$A22,Items!$F$2:$F$196,H$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$211,$A22,Items!$F$2:$F$211,H$5)</f>
         <v>0</v>
       </c>
       <c r="I22" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$196,$A22,Items!$G$2:$G$196,"Approved")</f>
+        <f>COUNTIFS(Items!$B$2:$B$211,$A22,Items!$G$2:$G$211,"Approved")</f>
         <v>0</v>
       </c>
       <c r="J22" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$196,$A22,Items!$G$2:$G$196,"Pending")</f>
+        <f>COUNTIFS(Items!$B$2:$B$211,$A22,Items!$G$2:$G$211,"Pending")</f>
         <v>6</v>
       </c>
       <c r="K22" s="4">
@@ -1134,44 +1134,44 @@
         </is>
       </c>
       <c r="B23" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$196,$A23)</f>
+        <f>COUNTIFS(Items!$B$2:$B$211,$A23)</f>
+        <v>23</v>
+      </c>
+      <c r="C23" s="0">
+        <f>COUNTIFS(Items!$B$2:$B$211,$A23,Items!$F$2:$F$211,C$5)</f>
         <v>22</v>
       </c>
-      <c r="C23" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$196,$A23,Items!$F$2:$F$196,C$5)</f>
-        <v>21</v>
-      </c>
       <c r="D23" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$196,$A23,Items!$F$2:$F$196,D$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$211,$A23,Items!$F$2:$F$211,D$5)</f>
         <v>0</v>
       </c>
       <c r="E23" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$196,$A23,Items!$F$2:$F$196,E$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$211,$A23,Items!$F$2:$F$211,E$5)</f>
         <v>0</v>
       </c>
       <c r="F23" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$196,$A23,Items!$F$2:$F$196,F$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$211,$A23,Items!$F$2:$F$211,F$5)</f>
         <v>1</v>
       </c>
       <c r="G23" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$196,$A23,Items!$F$2:$F$196,G$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$211,$A23,Items!$F$2:$F$211,G$5)</f>
         <v>0</v>
       </c>
       <c r="H23" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$196,$A23,Items!$F$2:$F$196,H$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$211,$A23,Items!$F$2:$F$211,H$5)</f>
         <v>0</v>
       </c>
       <c r="I23" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$196,$A23,Items!$G$2:$G$196,"Approved")</f>
+        <f>COUNTIFS(Items!$B$2:$B$211,$A23,Items!$G$2:$G$211,"Approved")</f>
         <v>0</v>
       </c>
       <c r="J23" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$196,$A23,Items!$G$2:$G$196,"Pending")</f>
-        <v>22</v>
+        <f>COUNTIFS(Items!$B$2:$B$211,$A23,Items!$G$2:$G$211,"Pending")</f>
+        <v>23</v>
       </c>
       <c r="K23" s="4">
         <f>IF(B23-G23=0,0,(D23+E23+F23)/(B23-G23))</f>
-        <v>0.045455</v>
+        <v>0.043478</v>
       </c>
       <c r="L23" s="4">
         <f>IF(B23-G23=0,0,H23/(B23-G23))</f>
@@ -1185,40 +1185,40 @@
         </is>
       </c>
       <c r="B24" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$196,$A24)</f>
-        <v>3</v>
+        <f>COUNTIFS(Items!$B$2:$B$211,$A24)</f>
+        <v>4</v>
       </c>
       <c r="C24" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$196,$A24,Items!$F$2:$F$196,C$5)</f>
-        <v>1</v>
+        <f>COUNTIFS(Items!$B$2:$B$211,$A24,Items!$F$2:$F$211,C$5)</f>
+        <v>2</v>
       </c>
       <c r="D24" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$196,$A24,Items!$F$2:$F$196,D$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$211,$A24,Items!$F$2:$F$211,D$5)</f>
         <v>0</v>
       </c>
       <c r="E24" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$196,$A24,Items!$F$2:$F$196,E$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$211,$A24,Items!$F$2:$F$211,E$5)</f>
         <v>0</v>
       </c>
       <c r="F24" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$196,$A24,Items!$F$2:$F$196,F$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$211,$A24,Items!$F$2:$F$211,F$5)</f>
         <v>0</v>
       </c>
       <c r="G24" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$196,$A24,Items!$F$2:$F$196,G$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$211,$A24,Items!$F$2:$F$211,G$5)</f>
         <v>2</v>
       </c>
       <c r="H24" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$196,$A24,Items!$F$2:$F$196,H$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$211,$A24,Items!$F$2:$F$211,H$5)</f>
         <v>0</v>
       </c>
       <c r="I24" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$196,$A24,Items!$G$2:$G$196,"Approved")</f>
+        <f>COUNTIFS(Items!$B$2:$B$211,$A24,Items!$G$2:$G$211,"Approved")</f>
         <v>0</v>
       </c>
       <c r="J24" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$196,$A24,Items!$G$2:$G$196,"Pending")</f>
-        <v>3</v>
+        <f>COUNTIFS(Items!$B$2:$B$211,$A24,Items!$G$2:$G$211,"Pending")</f>
+        <v>4</v>
       </c>
       <c r="K24" s="4">
         <f>IF(B24-G24=0,0,(D24+E24+F24)/(B24-G24))</f>
@@ -1236,40 +1236,40 @@
         </is>
       </c>
       <c r="B25" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$196,$A25)</f>
-        <v>3</v>
+        <f>COUNTIFS(Items!$B$2:$B$211,$A25)</f>
+        <v>8</v>
       </c>
       <c r="C25" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$196,$A25,Items!$F$2:$F$196,C$5)</f>
-        <v>2</v>
+        <f>COUNTIFS(Items!$B$2:$B$211,$A25,Items!$F$2:$F$211,C$5)</f>
+        <v>7</v>
       </c>
       <c r="D25" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$196,$A25,Items!$F$2:$F$196,D$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$211,$A25,Items!$F$2:$F$211,D$5)</f>
         <v>0</v>
       </c>
       <c r="E25" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$196,$A25,Items!$F$2:$F$196,E$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$211,$A25,Items!$F$2:$F$211,E$5)</f>
         <v>0</v>
       </c>
       <c r="F25" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$196,$A25,Items!$F$2:$F$196,F$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$211,$A25,Items!$F$2:$F$211,F$5)</f>
         <v>0</v>
       </c>
       <c r="G25" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$196,$A25,Items!$F$2:$F$196,G$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$211,$A25,Items!$F$2:$F$211,G$5)</f>
         <v>1</v>
       </c>
       <c r="H25" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$196,$A25,Items!$F$2:$F$196,H$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$211,$A25,Items!$F$2:$F$211,H$5)</f>
         <v>0</v>
       </c>
       <c r="I25" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$196,$A25,Items!$G$2:$G$196,"Approved")</f>
+        <f>COUNTIFS(Items!$B$2:$B$211,$A25,Items!$G$2:$G$211,"Approved")</f>
         <v>0</v>
       </c>
       <c r="J25" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$196,$A25,Items!$G$2:$G$196,"Pending")</f>
-        <v>3</v>
+        <f>COUNTIFS(Items!$B$2:$B$211,$A25,Items!$G$2:$G$211,"Pending")</f>
+        <v>8</v>
       </c>
       <c r="K25" s="4">
         <f>IF(B25-G25=0,0,(D25+E25+F25)/(B25-G25))</f>
@@ -1287,39 +1287,39 @@
         </is>
       </c>
       <c r="B26" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$196,$A26)</f>
+        <f>COUNTIFS(Items!$B$2:$B$211,$A26)</f>
         <v>3</v>
       </c>
       <c r="C26" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$196,$A26,Items!$F$2:$F$196,C$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$211,$A26,Items!$F$2:$F$211,C$5)</f>
         <v>3</v>
       </c>
       <c r="D26" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$196,$A26,Items!$F$2:$F$196,D$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$211,$A26,Items!$F$2:$F$211,D$5)</f>
         <v>0</v>
       </c>
       <c r="E26" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$196,$A26,Items!$F$2:$F$196,E$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$211,$A26,Items!$F$2:$F$211,E$5)</f>
         <v>0</v>
       </c>
       <c r="F26" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$196,$A26,Items!$F$2:$F$196,F$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$211,$A26,Items!$F$2:$F$211,F$5)</f>
         <v>0</v>
       </c>
       <c r="G26" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$196,$A26,Items!$F$2:$F$196,G$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$211,$A26,Items!$F$2:$F$211,G$5)</f>
         <v>0</v>
       </c>
       <c r="H26" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$196,$A26,Items!$F$2:$F$196,H$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$211,$A26,Items!$F$2:$F$211,H$5)</f>
         <v>0</v>
       </c>
       <c r="I26" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$196,$A26,Items!$G$2:$G$196,"Approved")</f>
+        <f>COUNTIFS(Items!$B$2:$B$211,$A26,Items!$G$2:$G$211,"Approved")</f>
         <v>0</v>
       </c>
       <c r="J26" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$196,$A26,Items!$G$2:$G$196,"Pending")</f>
+        <f>COUNTIFS(Items!$B$2:$B$211,$A26,Items!$G$2:$G$211,"Pending")</f>
         <v>3</v>
       </c>
       <c r="K26" s="4">
@@ -1338,40 +1338,40 @@
         </is>
       </c>
       <c r="B27" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$196,$A27)</f>
-        <v>12</v>
+        <f>COUNTIFS(Items!$B$2:$B$211,$A27)</f>
+        <v>14</v>
       </c>
       <c r="C27" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$196,$A27,Items!$F$2:$F$196,C$5)</f>
-        <v>12</v>
+        <f>COUNTIFS(Items!$B$2:$B$211,$A27,Items!$F$2:$F$211,C$5)</f>
+        <v>14</v>
       </c>
       <c r="D27" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$196,$A27,Items!$F$2:$F$196,D$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$211,$A27,Items!$F$2:$F$211,D$5)</f>
         <v>0</v>
       </c>
       <c r="E27" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$196,$A27,Items!$F$2:$F$196,E$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$211,$A27,Items!$F$2:$F$211,E$5)</f>
         <v>0</v>
       </c>
       <c r="F27" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$196,$A27,Items!$F$2:$F$196,F$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$211,$A27,Items!$F$2:$F$211,F$5)</f>
         <v>0</v>
       </c>
       <c r="G27" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$196,$A27,Items!$F$2:$F$196,G$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$211,$A27,Items!$F$2:$F$211,G$5)</f>
         <v>0</v>
       </c>
       <c r="H27" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$196,$A27,Items!$F$2:$F$196,H$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$211,$A27,Items!$F$2:$F$211,H$5)</f>
         <v>0</v>
       </c>
       <c r="I27" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$196,$A27,Items!$G$2:$G$196,"Approved")</f>
+        <f>COUNTIFS(Items!$B$2:$B$211,$A27,Items!$G$2:$G$211,"Approved")</f>
         <v>0</v>
       </c>
       <c r="J27" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$196,$A27,Items!$G$2:$G$196,"Pending")</f>
-        <v>12</v>
+        <f>COUNTIFS(Items!$B$2:$B$211,$A27,Items!$G$2:$G$211,"Pending")</f>
+        <v>14</v>
       </c>
       <c r="K27" s="4">
         <f>IF(B27-G27=0,0,(D27+E27+F27)/(B27-G27))</f>
@@ -1390,11 +1390,11 @@
       </c>
       <c r="B28" s="5">
         <f>SUM(B6:B27)</f>
-        <v>195</v>
+        <v>210</v>
       </c>
       <c r="C28" s="5">
         <f>SUM(C6:C27)</f>
-        <v>189</v>
+        <v>204</v>
       </c>
       <c r="D28" s="5">
         <f>SUM(D6:D27)</f>
@@ -1422,11 +1422,11 @@
       </c>
       <c r="J28" s="5">
         <f>SUM(J6:J27)</f>
-        <v>195</v>
+        <v>210</v>
       </c>
       <c r="K28" s="4">
         <f>IF(B28-G28=0,0,(D28+E28+F28)/(B28-G28))</f>
-        <v>0.015385</v>
+        <v>0.014286</v>
       </c>
       <c r="L28" s="4">
         <f>IF(B28-G28=0,0,H28/(B28-G28))</f>
@@ -1452,7 +1452,7 @@
         </is>
       </c>
       <c r="B31" s="0">
-        <f>COUNTIFS(Items!$F$2:$F$196,"Failed")</f>
+        <f>COUNTIFS(Items!$F$2:$F$211,"Failed")</f>
         <v>0</v>
       </c>
     </row>
@@ -1463,7 +1463,7 @@
         </is>
       </c>
       <c r="B32" s="0">
-        <f>COUNTIFS(Items!$F$2:$F$196,"Needs improvement")</f>
+        <f>COUNTIFS(Items!$F$2:$F$211,"Needs improvement")</f>
         <v>3</v>
       </c>
     </row>
@@ -1474,7 +1474,7 @@
         </is>
       </c>
       <c r="B33" s="0">
-        <f>COUNTIFS(Items!$F$2:$F$196,"Blocked")</f>
+        <f>COUNTIFS(Items!$F$2:$F$211,"Blocked")</f>
         <v>3</v>
       </c>
     </row>
@@ -1485,8 +1485,8 @@
         </is>
       </c>
       <c r="B34" s="0">
-        <f>COUNTIFS(Items!$L$2:$L$196,"&lt;&gt;",Items!$F$2:$F$196,"&lt;&gt;Passed")</f>
-        <v>7</v>
+        <f>COUNTIFS(Items!$L$2:$L$211,"&lt;&gt;",Items!$F$2:$F$211,"&lt;&gt;Passed")</f>
+        <v>11</v>
       </c>
     </row>
     <row r="35">
@@ -1496,8 +1496,8 @@
         </is>
       </c>
       <c r="B35" s="0">
-        <f>COUNTIFS(Items!$H$2:$H$196,"&lt;&gt;")</f>
-        <v>55</v>
+        <f>COUNTIFS(Items!$H$2:$H$211,"&lt;&gt;")</f>
+        <v>70</v>
       </c>
     </row>
   </sheetData>
@@ -3292,7 +3292,7 @@
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">The module badge aligns with the first line of the role description; long descriptions wrap below it; the top-right actions stay at the top; cards in one row keep one height with bottom-aligned actions; correct in both themes and at 375, 800, 1280 and 1600 px.</t>
+          <t xml:space="preserve">The module pill, description and actions share one centered line of one height for every card; the description ends in an ellipsis when it does not fit (see R81-10); correct in both themes and at 320, 375, 800, 1280 and 1600 px.</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
@@ -3327,7 +3327,7 @@
       </c>
       <c r="K19" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Root cause: a later override centred the badge against the whole multiline description and let the actions wrap below it. Fixed with first-baseline alignment (R8 phase 1).</t>
+          <t xml:space="preserve">Root cause: a later override centred the badge against the whole multiline description and let the actions wrap below it. Fixed with first-baseline alignment (R8 phase 1). Superseded in R8 addendum: the header no longer wraps; the full description is available on demand (R81-10).</t>
         </is>
       </c>
       <c r="L19" s="2" t="inlineStr">
@@ -20011,7 +20011,7 @@
       </c>
       <c r="K191" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">No throttling of failed Basic logins; group-readable secret files are accepted (documented limitations).</t>
+          <t xml:space="preserve">No throttling of failed Basic logins; group-readable secret files are accepted (documented limitations). Update R8.1: failed Basic sign-ins are throttled (R81-01) and group-readable secrets need an explicit opt-in (R81-02).</t>
         </is>
       </c>
       <c r="L191" s="2" t="inlineStr">
@@ -20021,7 +20021,7 @@
       </c>
       <c r="M191" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Throttle failed logins at the gateway or in the application, and reject group-readable secret files after a compatibility review of systemd and container secret mounts.</t>
+          <t xml:space="preserve">Share throttle state across workers if the runtime ever scales out.</t>
         </is>
       </c>
       <c r="N191" s="2" t="inlineStr">
@@ -20031,7 +20031,7 @@
       </c>
       <c r="O191" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Throttling and group permissions are open decisions (SECURITY_REVIEW_R8).</t>
+          <t xml:space="preserve">Throttling is per process (see R81-01); distributed guessing relies on the 32 character secret.</t>
         </is>
       </c>
       <c r="P191" s="2" t="inlineStr">
@@ -20535,6 +20535,1461 @@
         </is>
       </c>
       <c r="S196" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">R81-01</t>
+        </is>
+      </c>
+      <c r="B197" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Security and Data Integrity</t>
+        </is>
+      </c>
+      <c r="C197" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Server › Failed Basic sign-in throttling</t>
+        </is>
+      </c>
+      <c r="D197" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Repeated wrong Basic credentials from one client lock that client out with 429 and Retry-After (default 5 failures, 60 s, doubling to 15 min); correct credentials are refused during the lock-out and accepted after it; other clients, health probes and requests without credentials are unaffected; forwarded headers from an untrusted peer change nothing.</t>
+        </is>
+      </c>
+      <c r="E197" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">High</t>
+        </is>
+      </c>
+      <c r="F197" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not tested</t>
+        </is>
+      </c>
+      <c r="G197" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pending</t>
+        </is>
+      </c>
+      <c r="H197" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">backend/tests/test_auth_throttle.py; backend/tests/test_security_surface.py</t>
+        </is>
+      </c>
+      <c r="I197" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="J197" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="K197" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Implemented in R8.1 (SEC-02). Automated tests use a fake clock and a TestClient; no real network, proxy or multi-worker deployment was exercised.</t>
+        </is>
+      </c>
+      <c r="L197" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SEC-02</t>
+        </is>
+      </c>
+      <c r="M197" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Share counters between workers or hosts, or throttle per forwarded identity at the gateway.</t>
+        </is>
+      </c>
+      <c r="N197" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">On a test server with Basic authentication, send six wrong passwords from one browser, confirm the 429 page and wait the Retry-After time, then sign in; repeat behind your reverse proxy with SAP_LENS_TRUSTED_PROXIES set and confirm other users are not locked out.</t>
+        </is>
+      </c>
+      <c r="O197" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">State is per process and lost on restart; clients behind one NAT or an unlisted proxy share a lock-out; distributed guessing is slowed, not stopped.</t>
+        </is>
+      </c>
+      <c r="P197" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">docs/deployment/SECURITY.md; backend/deployment.py; backend/main.py</t>
+        </is>
+      </c>
+      <c r="Q197" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Implemented</t>
+        </is>
+      </c>
+      <c r="R197" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Unclassified</t>
+        </is>
+      </c>
+      <c r="S197" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">R81-02</t>
+        </is>
+      </c>
+      <c r="B198" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Security and Data Integrity</t>
+        </is>
+      </c>
+      <c r="C198" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Server › Access secret file permissions (Linux)</t>
+        </is>
+      </c>
+      <c r="D198" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A new secret is created owner-only (0600); an existing secret readable by other users, or writable or executable by its group, is refused; group read (0640) is accepted only with SAP_LENS_AUTH_SECRET_GROUP_READ=1 and a group the service account belongs to; every refusal names the file, its mode and the fix; the file is never changed.</t>
+        </is>
+      </c>
+      <c r="E198" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">High</t>
+        </is>
+      </c>
+      <c r="F198" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not tested</t>
+        </is>
+      </c>
+      <c r="G198" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pending</t>
+        </is>
+      </c>
+      <c r="H198" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">backend/tests/test_secret_file_policy.py; backend/tests/test_security_surface.py</t>
+        </is>
+      </c>
+      <c r="I198" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="J198" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="K198" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Implemented in R8.1 (SEC-03). Judged on the opened file; symlinks resolve to their target.</t>
+        </is>
+      </c>
+      <c r="L198" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SEC-03</t>
+        </is>
+      </c>
+      <c r="M198" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Verify the owner and effective access through the service account, not only the mode.</t>
+        </is>
+      </c>
+      <c r="N198" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">On a Linux host start the server with a 0644, a 0640 and a 0600 secret (with and without the opt-in) and read the messages; confirm the systemd service and the Docker compose installation still start.</t>
+        </is>
+      </c>
+      <c r="O198" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">An existing 0640 secret needs chmod 600 or the opt-in (migration step, documented). Not exercised under real systemd or Docker here.</t>
+        </is>
+      </c>
+      <c r="P198" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">docs/deployment/SECURITY.md; backend/deployment.py; backend/server.py; compose.yml</t>
+        </is>
+      </c>
+      <c r="Q198" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Implemented</t>
+        </is>
+      </c>
+      <c r="R198" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Unclassified</t>
+        </is>
+      </c>
+      <c r="S198" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">R81-03</t>
+        </is>
+      </c>
+      <c r="B199" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Server and Deployment</t>
+        </is>
+      </c>
+      <c r="C199" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Windows service › Secret file ACL</t>
+        </is>
+      </c>
+      <c r="D199" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The installed secret file grants access only to SYSTEM, Administrators and read access to the service account; a manually created secret with broader access is noticed by the administrator (the runtime does not verify an ACL).</t>
+        </is>
+      </c>
+      <c r="E199" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Medium</t>
+        </is>
+      </c>
+      <c r="F199" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not tested</t>
+        </is>
+      </c>
+      <c r="G199" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pending</t>
+        </is>
+      </c>
+      <c r="H199" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">backend/tests/test_deployment_contracts.py</t>
+        </is>
+      </c>
+      <c r="I199" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="J199" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="K199" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Provisioning applies the ACL with icacls (manage-server-service.ps1). Windows ACLs are not evaluated by the Linux tests and not checked at runtime.</t>
+        </is>
+      </c>
+      <c r="L199" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SEC-03</t>
+        </is>
+      </c>
+      <c r="M199" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Check the ACL at start (icacls or the Win32 API) and warn like the POSIX check.</t>
+        </is>
+      </c>
+      <c r="N199" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">On Windows run icacls on the secret after installation and after any manual replacement; start the service and sign in.</t>
+        </is>
+      </c>
+      <c r="O199" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Blocked on a Windows host: not run in this validation.</t>
+        </is>
+      </c>
+      <c r="P199" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">docs/deployment/WINDOWS_SERVICE.md; scripts/manage-server-service.ps1</t>
+        </is>
+      </c>
+      <c r="Q199" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Partially implemented</t>
+        </is>
+      </c>
+      <c r="R199" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Unclassified</t>
+        </is>
+      </c>
+      <c r="S199" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">R81-04</t>
+        </is>
+      </c>
+      <c r="B200" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SoD Reports</t>
+        </is>
+      </c>
+      <c r="C200" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SoD › Reports › PDF</t>
+        </is>
+      </c>
+      <c r="D200" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A PDF built from a review period lists risk names and descriptions in the findings section and activity names and descriptions in the appendices, each with its source (Imported, Local fallback or Not available) and a source legend; a file without descriptions produces the report as before.</t>
+        </is>
+      </c>
+      <c r="E200" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Medium</t>
+        </is>
+      </c>
+      <c r="F200" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not tested</t>
+        </is>
+      </c>
+      <c r="G200" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pending</t>
+        </is>
+      </c>
+      <c r="H200" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">backend/tests/test_sod_report_metadata.py; backend/tests/test_sod_reports.py</t>
+        </is>
+      </c>
+      <c r="I200" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="J200" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="K200" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Implemented in R8.1. Layout was checked through the model and file validity, not by looking at pages.</t>
+        </is>
+      </c>
+      <c r="L200" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="M200" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Show transaction descriptions with their source in the same tables.</t>
+        </is>
+      </c>
+      <c r="N200" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Generate a PDF for a period captured from a CSV with description columns and read the tables and legend; try a period captured before descriptions were retained.</t>
+        </is>
+      </c>
+      <c r="O200" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A description with characters outside the bundled PDF font fails the PDF with an explicit message (DOCX works).</t>
+        </is>
+      </c>
+      <c r="P200" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">docs/features/SOD.md; backend/sod_reports.py; backend/sod_metadata.py</t>
+        </is>
+      </c>
+      <c r="Q200" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Implemented</t>
+        </is>
+      </c>
+      <c r="R200" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Unclassified</t>
+        </is>
+      </c>
+      <c r="S200" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">R81-05</t>
+        </is>
+      </c>
+      <c r="B201" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SoD Reports</t>
+        </is>
+      </c>
+      <c r="C201" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SoD › Reports › DOCX</t>
+        </is>
+      </c>
+      <c r="D201" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The editable DOCX contains the same description tables, source labels and legend as the PDF, with special characters and long text intact and markup shown as text.</t>
+        </is>
+      </c>
+      <c r="E201" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Medium</t>
+        </is>
+      </c>
+      <c r="F201" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not tested</t>
+        </is>
+      </c>
+      <c r="G201" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pending</t>
+        </is>
+      </c>
+      <c r="H201" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">backend/tests/test_sod_report_metadata.py; backend/tests/test_sod_reports.py</t>
+        </is>
+      </c>
+      <c r="I201" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="J201" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="K201" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Implemented in R8.1; content checked in the document XML.</t>
+        </is>
+      </c>
+      <c r="L201" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="M201" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="N201" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Open the DOCX in Word and read the Source column, the legend and a long description.</t>
+        </is>
+      </c>
+      <c r="O201" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not opened in Word in this validation.</t>
+        </is>
+      </c>
+      <c r="P201" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">docs/features/SOD.md; backend/sod_reports.py</t>
+        </is>
+      </c>
+      <c r="Q201" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Implemented</t>
+        </is>
+      </c>
+      <c r="R201" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Unclassified</t>
+        </is>
+      </c>
+      <c r="S201" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">R81-06</t>
+        </is>
+      </c>
+      <c r="B202" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SoD Reports</t>
+        </is>
+      </c>
+      <c r="C202" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SoD › Reports › Description provenance</t>
+        </is>
+      </c>
+      <c r="D202" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Imported text wins, local business text is shown only where the import has none and is labelled Local fallback, a differing local text is reported but never mixed in, and nothing is generated for a missing description.</t>
+        </is>
+      </c>
+      <c r="E202" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">High</t>
+        </is>
+      </c>
+      <c r="F202" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not tested</t>
+        </is>
+      </c>
+      <c r="G202" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pending</t>
+        </is>
+      </c>
+      <c r="H202" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">backend/tests/test_sod_report_metadata.py; backend/tests/test_sod_metadata.py</t>
+        </is>
+      </c>
+      <c r="I202" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="J202" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="K202" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The report uses the resolver that also serves the pills and Settings.</t>
+        </is>
+      </c>
+      <c r="L202" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="M202" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="N202" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Compare one risk and one activity across the pill popover, Settings and the report.</t>
+        </is>
+      </c>
+      <c r="O202" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="P202" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">backend/sod_metadata.py; docs/data/SOD_MATRIX.md</t>
+        </is>
+      </c>
+      <c r="Q202" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Implemented</t>
+        </is>
+      </c>
+      <c r="R202" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Unclassified</t>
+        </is>
+      </c>
+      <c r="S202" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">R81-07</t>
+        </is>
+      </c>
+      <c r="B203" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Review Periods</t>
+        </is>
+      </c>
+      <c r="C203" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Review Periods › Frozen descriptions</t>
+        </is>
+      </c>
+      <c r="D203" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A period report never shows descriptions imported or edited after the period was captured; an approved period keeps its report model checksum; a period captured before R8.1 shows only its frozen local text and says that imported descriptions were not retained; decisions and approvals are unchanged.</t>
+        </is>
+      </c>
+      <c r="E203" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Critical</t>
+        </is>
+      </c>
+      <c r="F203" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not tested</t>
+        </is>
+      </c>
+      <c r="G203" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pending</t>
+        </is>
+      </c>
+      <c r="H203" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">backend/tests/test_sod_report_metadata.py; backend/tests/test_sod_periods_v2.py</t>
+        </is>
+      </c>
+      <c r="I203" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="J203" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="K203" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Descriptions are stored inside the immutable snapshot (metadata version 1).</t>
+        </is>
+      </c>
+      <c r="L203" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="M203" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="N203" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Approve a period, import a CSV with different descriptions, regenerate the report and compare; open a period created before the upgrade.</t>
+        </is>
+      </c>
+      <c r="O203" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Legacy snapshots cannot show imported descriptions; recapturing a period replaces its copy by design.</t>
+        </is>
+      </c>
+      <c r="P203" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">docs/features/SOD.md; backend/sod_periods.py</t>
+        </is>
+      </c>
+      <c r="Q203" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Implemented</t>
+        </is>
+      </c>
+      <c r="R203" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Unclassified</t>
+        </is>
+      </c>
+      <c r="S203" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">R81-08</t>
+        </is>
+      </c>
+      <c r="B204" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Settings and Data Sources</t>
+        </is>
+      </c>
+      <c r="C204" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SoD Matrix › Legacy files in reports</t>
+        </is>
+      </c>
+      <c r="D204" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A SoD Matrix CSV without any optional description column, or with partly filled ones, still imports, reviews and reports; missing descriptions never block a PDF or DOCX.</t>
+        </is>
+      </c>
+      <c r="E204" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">High</t>
+        </is>
+      </c>
+      <c r="F204" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not tested</t>
+        </is>
+      </c>
+      <c r="G204" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pending</t>
+        </is>
+      </c>
+      <c r="H204" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">backend/tests/test_sod_report_metadata.py; backend/tests/test_sod_metadata.py</t>
+        </is>
+      </c>
+      <c r="I204" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="J204" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="K204" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Old datasets produce the report tables they always did.</t>
+        </is>
+      </c>
+      <c r="L204" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="M204" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="N204" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Run the report on your existing production-shaped export.</t>
+        </is>
+      </c>
+      <c r="O204" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No real upstream export was available.</t>
+        </is>
+      </c>
+      <c r="P204" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">docs/data/SOD_MATRIX.md</t>
+        </is>
+      </c>
+      <c r="Q204" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Implemented</t>
+        </is>
+      </c>
+      <c r="R204" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Unclassified</t>
+        </is>
+      </c>
+      <c r="S204" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">R81-09</t>
+        </is>
+      </c>
+      <c r="B205" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Component Library</t>
+        </is>
+      </c>
+      <c r="C205" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Components › Select dropdown family</t>
+        </is>
+      </c>
+      <c r="D205" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Standard selects, the searchable select and the multi-select filter open the same list surface (background, border, radius, spacing, hover, accent and check mark for the selected option); long labels wrap, disabled options cannot be chosen, the list stays inside the viewport and above dialogs and side panels, and works with mouse, keyboard, Escape and screen readers, in both themes.</t>
+        </is>
+      </c>
+      <c r="E205" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">High</t>
+        </is>
+      </c>
+      <c r="F205" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not tested</t>
+        </is>
+      </c>
+      <c r="G205" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pending</t>
+        </is>
+      </c>
+      <c r="H205" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">frontend/tests/select-family.spec.ts; frontend/tests/a11y-audit.spec.ts</t>
+        </is>
+      </c>
+      <c r="I205" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="J205" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="K205" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Implemented as an addendum to R8; the native select element is kept for value, validation and labels.</t>
+        </is>
+      </c>
+      <c r="L205" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="M205" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="N205" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Open Component Library › Demo select, Demo searchable role and Demo areas in light and dark at 375, 800, 1280 and 1600 px and compare them; try the selects inside the demo dialog and side panel and a screen reader.</t>
+        </is>
+      </c>
+      <c r="O205" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Multiple or sized selects keep the browser control; not tried with a screen reader or on a touch device.</t>
+        </is>
+      </c>
+      <c r="P205" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">docs/architecture/COMPONENTS.md; frontend/src/components/Shared/Select.tsx</t>
+        </is>
+      </c>
+      <c r="Q205" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Implemented</t>
+        </is>
+      </c>
+      <c r="R205" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Unclassified</t>
+        </is>
+      </c>
+      <c r="S205" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">R81-10</t>
+        </is>
+      </c>
+      <c r="B206" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Role Lookup</t>
+        </is>
+      </c>
+      <c r="C206" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Role Lookup › Card header description</t>
+        </is>
+      </c>
+      <c r="D206" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The module pill, description and actions share one centered line of one height for every card; a description that does not fit ends in an ellipsis and reveals its full text on hover, keyboard focus, click or tap; a description that fits has no control and no tooltip; actions never shrink; correct with long English and French text, at 320 to 1600 px and in both themes.</t>
+        </is>
+      </c>
+      <c r="E206" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Medium</t>
+        </is>
+      </c>
+      <c r="F206" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not tested</t>
+        </is>
+      </c>
+      <c r="G206" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pending</t>
+        </is>
+      </c>
+      <c r="H206" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">frontend/tests/r8-ui-polish.spec.ts; frontend/tests/a11y-audit.spec.ts</t>
+        </is>
+      </c>
+      <c r="I206" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="J206" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="K206" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Addendum to R8-01 (which described the earlier wrapping header). The visible part is short at 375 px by design; the full text is on demand.</t>
+        </is>
+      </c>
+      <c r="L206" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="M206" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="N206" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Resize the browser and zoom to 200 and 400 percent on Role Lookup with long descriptions, in both themes.</t>
+        </is>
+      </c>
+      <c r="O206" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">At 375 px or less only a few characters of the description remain visible beside the pill and two actions.</t>
+        </is>
+      </c>
+      <c r="P206" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">docs/architecture/COMPONENTS.md; frontend/src/components/Shared/TruncatedText.tsx</t>
+        </is>
+      </c>
+      <c r="Q206" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Implemented</t>
+        </is>
+      </c>
+      <c r="R206" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Unclassified</t>
+        </is>
+      </c>
+      <c r="S206" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">R81-11</t>
+        </is>
+      </c>
+      <c r="B207" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Server and Deployment</t>
+        </is>
+      </c>
+      <c r="C207" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Repository › Ruff and ESLint</t>
+        </is>
+      </c>
+      <c r="D207" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ruff and ESLint run in Fast Validation, Full Validation and the local profiles, fail on errors and on new ESLint warnings beyond the recorded backlog, and a documented command reproduces each.</t>
+        </is>
+      </c>
+      <c r="E207" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Medium</t>
+        </is>
+      </c>
+      <c r="F207" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not tested</t>
+        </is>
+      </c>
+      <c r="G207" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pending</t>
+        </is>
+      </c>
+      <c r="H207" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">backend/tests/test_workflows.py; backend/tests/test_test_profiles.py</t>
+        </is>
+      </c>
+      <c r="I207" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="J207" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="K207" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Correctness rules only; no reformatting.</t>
+        </is>
+      </c>
+      <c r="L207" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="M207" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="N207" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Run python -m ruff check backend scripts and npm run lint in frontend; read the Fast Validation summary on GitHub.</t>
+        </is>
+      </c>
+      <c r="O207" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ESLint backlog: 30 hook-dependency warnings and 81 any uses in specs.</t>
+        </is>
+      </c>
+      <c r="P207" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">docs/development/TESTING.md; ruff.toml; frontend/eslint.config.js</t>
+        </is>
+      </c>
+      <c r="Q207" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Implemented</t>
+        </is>
+      </c>
+      <c r="R207" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Unclassified</t>
+        </is>
+      </c>
+      <c r="S207" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">R81-12</t>
+        </is>
+      </c>
+      <c r="B208" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Server and Deployment</t>
+        </is>
+      </c>
+      <c r="C208" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Repository › Test process isolation</t>
+        </is>
+      </c>
+      <c r="D208" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Browser test servers remove their temporary directories when stopped, the runner reports busy ports instead of colliding and stops only processes it started.</t>
+        </is>
+      </c>
+      <c r="E208" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Medium</t>
+        </is>
+      </c>
+      <c r="F208" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not tested</t>
+        </is>
+      </c>
+      <c r="G208" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pending</t>
+        </is>
+      </c>
+      <c r="H208" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">backend/tests/test_test_profiles.py</t>
+        </is>
+      </c>
+      <c r="I208" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="J208" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="K208" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Found 616 leaked directories (1.9 GB) before the fix.</t>
+        </is>
+      </c>
+      <c r="L208" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="M208" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="N208" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Run a browser spec and check that no sap-lens-browser-* directory and no server process remain.</t>
+        </is>
+      </c>
+      <c r="O208" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="P208" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">docs/development/TESTING.md; scripts/serve-browser-tests.py; scripts/run-tests.py</t>
+        </is>
+      </c>
+      <c r="Q208" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Implemented</t>
+        </is>
+      </c>
+      <c r="R208" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Unclassified</t>
+        </is>
+      </c>
+      <c r="S208" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">R81-13</t>
+        </is>
+      </c>
+      <c r="B209" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Server and Deployment</t>
+        </is>
+      </c>
+      <c r="C209" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Repository › Parallel regression</t>
+        </is>
+      </c>
+      <c r="D209" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The regression runs the browser suite in up to three isolated processes with deterministic distribution, per-process attribution and the same results as a serial run.</t>
+        </is>
+      </c>
+      <c r="E209" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Medium</t>
+        </is>
+      </c>
+      <c r="F209" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not tested</t>
+        </is>
+      </c>
+      <c r="G209" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pending</t>
+        </is>
+      </c>
+      <c r="H209" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">backend/tests/test_test_profiles.py</t>
+        </is>
+      </c>
+      <c r="I209" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="J209" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="K209" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">See R8_1_STABILIZATION.md for the measurements and the one load-dependent failure observed.</t>
+        </is>
+      </c>
+      <c r="L209" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="M209" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="N209" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Run regression --browser-jobs auto on a 4 CPU host and compare with --browser-jobs 1 when a result is doubtful.</t>
+        </is>
+      </c>
+      <c r="O209" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CPU-bound: gains were 1.6x to 1.7x on 4 vCPUs; not measured on CI runners.</t>
+        </is>
+      </c>
+      <c r="P209" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">docs/development/TESTING.md; docs/development/R8_1_STABILIZATION.md</t>
+        </is>
+      </c>
+      <c r="Q209" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Implemented</t>
+        </is>
+      </c>
+      <c r="R209" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Unclassified</t>
+        </is>
+      </c>
+      <c r="S209" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">R81-14</t>
+        </is>
+      </c>
+      <c r="B210" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Desktop and Startup</t>
+        </is>
+      </c>
+      <c r="C210" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Windows desktop and service › R8.1 changes</t>
+        </is>
+      </c>
+      <c r="D210" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">On Windows the desktop application, the server mode with Basic authentication (throttling, secret ACL) and the Windows service start, sign in, lock out and recover as documented, and the select dropdowns, truncated descriptions and report descriptions work in WebView2.</t>
+        </is>
+      </c>
+      <c r="E210" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">High</t>
+        </is>
+      </c>
+      <c r="F210" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not tested</t>
+        </is>
+      </c>
+      <c r="G210" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pending</t>
+        </is>
+      </c>
+      <c r="H210" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">backend/tests/test_deployment_contracts.py; backend/tests/test_desktop.py</t>
+        </is>
+      </c>
+      <c r="I210" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="J210" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="K210" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Native Windows, WebView2, service control and installer behaviour were not validated.</t>
+        </is>
+      </c>
+      <c r="L210" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="M210" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="N210" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Install the desktop build and the service on Windows 11 at 100, 150 and 200 percent scaling and walk the R81 items.</t>
+        </is>
+      </c>
+      <c r="O210" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Blocked here: no Windows host.</t>
+        </is>
+      </c>
+      <c r="P210" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">docs/deployment/WINDOWS_SERVICE.md; docs/architecture/DESKTOP.md</t>
+        </is>
+      </c>
+      <c r="Q210" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Partially implemented</t>
+        </is>
+      </c>
+      <c r="R210" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Unclassified</t>
+        </is>
+      </c>
+      <c r="S210" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">R81-15</t>
+        </is>
+      </c>
+      <c r="B211" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Server and Deployment</t>
+        </is>
+      </c>
+      <c r="C211" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Docker and systemd › R8.1 changes</t>
+        </is>
+      </c>
+      <c r="D211" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The Docker installation (0640 secret with the explicit opt-in) and the hardened systemd unit (seven added sandbox directives) start, serve and restart on real hosts.</t>
+        </is>
+      </c>
+      <c r="E211" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">High</t>
+        </is>
+      </c>
+      <c r="F211" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not tested</t>
+        </is>
+      </c>
+      <c r="G211" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pending</t>
+        </is>
+      </c>
+      <c r="H211" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">backend/tests/test_deployment_contracts.py; backend/tests/test_server.py</t>
+        </is>
+      </c>
+      <c r="I211" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="J211" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="K211" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The unit passed systemd-analyze verify; it was not booted. Docker was not run.</t>
+        </is>
+      </c>
+      <c r="L211" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SEC-07</t>
+        </is>
+      </c>
+      <c r="M211" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="N211" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Install both on a test host, check journalctl or docker logs, sign in, restart.</t>
+        </is>
+      </c>
+      <c r="O211" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Blocked here: no real systemd or Docker runtime.</t>
+        </is>
+      </c>
+      <c r="P211" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">docs/deployment/LINUX_DOCKER.md; docs/deployment/LINUX_NATIVE.md; deploy/linux/sap-lens.service</t>
+        </is>
+      </c>
+      <c r="Q211" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Partially implemented</t>
+        </is>
+      </c>
+      <c r="R211" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Unclassified</t>
+        </is>
+      </c>
+      <c r="S211" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Not started</t>
         </is>
@@ -21069,12 +22524,12 @@
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">No throttling of failed Basic logins; group-readable secret files are accepted (documented limitations).</t>
+          <t xml:space="preserve">No throttling of failed Basic logins; group-readable secret files are accepted (documented limitations). Update R8.1: failed Basic sign-ins are throttled (R81-01) and group-readable secrets need an explicit opt-in (R81-02).</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Throttling and group permissions are open decisions (SECURITY_REVIEW_R8).</t>
+          <t xml:space="preserve">Throttling is per process (see R81-01); distributed guessing relies on the 32 character secret.</t>
         </is>
       </c>
     </row>
@@ -21204,8 +22659,176 @@
         </is>
       </c>
     </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">R81-01</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Security and Data Integrity</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Server › Failed Basic sign-in throttling</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">High</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not tested</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SEC-02</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Implemented in R8.1 (SEC-02). Automated tests use a fake clock and a TestClient; no real network, proxy or multi-worker deployment was exercised.</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">State is per process and lost on restart; clients behind one NAT or an unlisted proxy share a lock-out; distributed guessing is slowed, not stopped.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">R81-02</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Security and Data Integrity</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Server › Access secret file permissions (Linux)</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">High</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not tested</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SEC-03</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Implemented in R8.1 (SEC-03). Judged on the opened file; symlinks resolve to their target.</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">An existing 0640 secret needs chmod 600 or the opt-in (migration step, documented). Not exercised under real systemd or Docker here.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">R81-03</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Server and Deployment</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Windows service › Secret file ACL</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Medium</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not tested</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SEC-03</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Provisioning applies the ACL with icacls (manage-server-service.ps1). Windows ACLs are not evaluated by the Linux tests and not checked at runtime.</t>
+        </is>
+      </c>
+      <c r="H17" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Blocked on a Windows host: not run in this validation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">R81-15</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Server and Deployment</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Docker and systemd › R8.1 changes</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">High</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not tested</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SEC-07</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The unit passed systemd-analyze verify; it was not booted. Docker was not run.</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Blocked here: no real systemd or Docker runtime.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:H14"/>
+  <autoFilter ref="A1:H18"/>
   <conditionalFormatting sqref="E2:E2000">
     <cfRule type="cellIs" dxfId="0" priority="1" operator="equal">
       <formula>"Passed"</formula>
@@ -21488,12 +23111,12 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Throttle failed logins at the gateway or in the application, and reject group-readable secret files after a compatibility review of systemd and container secret mounts.</t>
+          <t xml:space="preserve">Share throttle state across workers if the runtime ever scales out.</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">No throttling of failed Basic logins; group-readable secret files are accepted (documented limitations).</t>
+          <t xml:space="preserve">No throttling of failed Basic logins; group-readable secret files are accepted (documented limitations). Update R8.1: failed Basic sign-ins are throttled (R81-01) and group-readable secrets need an explicit opt-in (R81-02).</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
@@ -21586,8 +23209,176 @@
         </is>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">R81-01</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Security and Data Integrity</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Server › Failed Basic sign-in throttling</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">High</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not tested</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Share counters between workers or hosts, or throttle per forwarded identity at the gateway.</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Implemented in R8.1 (SEC-02). Automated tests use a fake clock and a TestClient; no real network, proxy or multi-worker deployment was exercised.</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SEC-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">R81-02</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Security and Data Integrity</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Server › Access secret file permissions (Linux)</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">High</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not tested</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Verify the owner and effective access through the service account, not only the mode.</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Implemented in R8.1 (SEC-03). Judged on the opened file; symlinks resolve to their target.</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SEC-03</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">R81-03</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Server and Deployment</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Windows service › Secret file ACL</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Medium</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not tested</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Check the ACL at start (icacls or the Win32 API) and warn like the POSIX check.</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Provisioning applies the ACL with icacls (manage-server-service.ps1). Windows ACLs are not evaluated by the Linux tests and not checked at runtime.</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SEC-03</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">R81-04</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SoD Reports</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SoD › Reports › PDF</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Medium</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not tested</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Show transaction descriptions with their source in the same tables.</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Implemented in R8.1. Layout was checked through the model and file validity, not by looking at pages.</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:H8"/>
+  <autoFilter ref="A1:H12"/>
   <conditionalFormatting sqref="E2:E2000">
     <cfRule type="cellIs" dxfId="0" priority="1" operator="equal">
       <formula>"Passed"</formula>

</xml_diff>

<commit_message>
refactor(ci): one build_target dropdown replaces the operating system and package inputs
GitHub cannot make one choice depend on another, so the package list showed
incompatible options. The Build Deployment Packages workflow now has a single
build_target choice (all, windows-all, windows-desktop, windows-service,
linux-all, linux-docker, linux-native); every value is valid and the combination
validation is gone. The planning job resolves it once, rejects only an unknown
value before any expensive job, and the run summary shows the target and the
resolved packages. Package jobs, skipped-job handling, artifact names, versioning,
channels, verification and publication gating (planned, selected and verified
packages only) are unchanged. Covered offline; no workflow was dispatched.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EsCXzFEofbBScBiLBFpRK2
</commit_message>
<xml_diff>
--- a/docs/validation/validation-tracker.xlsx
+++ b/docs/validation/validation-tracker.xlsx
@@ -22013,7 +22013,7 @@
       </c>
       <c r="D212" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">The operating system (all, windows, linux) and package (all or one) inputs build exactly the documented packages; an incompatible pair fails in the first job before validation or any packaging runner starts; unselected packages are skipped and start no runner; the summary lists every package as selected or skipped; publication takes only selected, verified packages and is never blocked or widened by skipped ones.</t>
+          <t xml:space="preserve">GitHub Actions shows one build_target dropdown (all, windows-all, windows-desktop, windows-service, linux-all, linux-docker, linux-native) and every choice is valid; the selected packages are built independently, unselected packages are skipped and start no runner, the summary shows the target and resolved packages, and publication takes only selected, verified packages and is never blocked or widened by skipped ones.</t>
         </is>
       </c>
       <c r="E212" s="2" t="inlineStr">
@@ -22048,7 +22048,7 @@
       </c>
       <c r="K212" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Implemented as an R8.1 follow-up. Verified offline: planner, resolver, workflow job conditions and publication gating; no workflow was dispatched.</t>
+          <t xml:space="preserve">Implemented as an R8.1 follow-up; a two-input version (operating_system and package) was replaced by the single dropdown because incompatible choices could not be hidden. Verified offline: planner, resolver, workflow job conditions and publication gating; no workflow was dispatched.</t>
         </is>
       </c>
       <c r="L212" s="2" t="inlineStr">
@@ -22063,7 +22063,7 @@
       </c>
       <c r="N212" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">After approval, dispatch a build-only run for windows/all, linux/all and one rejected pair (windows with linux-docker) and read the Resolve Build Selection summary; check that skipped jobs start no runner.</t>
+          <t xml:space="preserve">After approval, dispatch build-only runs for windows-all, linux-all and one single package and read the Resolve Build Selection summary; check that skipped jobs start no runner and that the dropdown shows exactly seven choices.</t>
         </is>
       </c>
       <c r="O212" s="2" t="inlineStr">

</xml_diff>

<commit_message>
feat(ci): release failure-handling tests, Stable-from-main rule, workflow matrix and tracker items
- Stable / Production publication is refused unless the run is on main, in the
  plan job (before any runner is spent) and again at publication
- Tests: missing or corrupted artifact, failed smoke test, cancelled run,
  missing publish switch or environment, build-only needs no publication rights
- Contract: publication must run in a protected environment (clear error)
- docs: workflow validation matrix with run evidence, runtime validation plan,
  workflow security audit in CI_CD.md
- tracker: CICD-01..13 (all Not tested / Pending), workbook regenerated

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EsCXzFEofbBScBiLBFpRK2
</commit_message>
<xml_diff>
--- a/docs/validation/validation-tracker.xlsx
+++ b/docs/validation/validation-tracker.xlsx
@@ -133,8 +133,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ValidationItems" displayName="ValidationItems" ref="A1:S212" totalsRowShown="0">
-  <autoFilter ref="A1:S212"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ValidationItems" displayName="ValidationItems" ref="A1:S225" totalsRowShown="0">
+  <autoFilter ref="A1:S225"/>
   <tableColumns count="19">
     <tableColumn id="1" name="ID"/>
     <tableColumn id="2" name="Area"/>
@@ -267,39 +267,39 @@
         </is>
       </c>
       <c r="B6" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$212,$A6)</f>
+        <f>COUNTIFS(Items!$B$2:$B$225,$A6)</f>
         <v>9</v>
       </c>
       <c r="C6" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$212,$A6,Items!$F$2:$F$212,C$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$225,$A6,Items!$F$2:$F$225,C$5)</f>
         <v>9</v>
       </c>
       <c r="D6" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$212,$A6,Items!$F$2:$F$212,D$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$225,$A6,Items!$F$2:$F$225,D$5)</f>
         <v>0</v>
       </c>
       <c r="E6" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$212,$A6,Items!$F$2:$F$212,E$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$225,$A6,Items!$F$2:$F$225,E$5)</f>
         <v>0</v>
       </c>
       <c r="F6" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$212,$A6,Items!$F$2:$F$212,F$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$225,$A6,Items!$F$2:$F$225,F$5)</f>
         <v>0</v>
       </c>
       <c r="G6" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$212,$A6,Items!$F$2:$F$212,G$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$225,$A6,Items!$F$2:$F$225,G$5)</f>
         <v>0</v>
       </c>
       <c r="H6" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$212,$A6,Items!$F$2:$F$212,H$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$225,$A6,Items!$F$2:$F$225,H$5)</f>
         <v>0</v>
       </c>
       <c r="I6" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$212,$A6,Items!$G$2:$G$212,"Approved")</f>
+        <f>COUNTIFS(Items!$B$2:$B$225,$A6,Items!$G$2:$G$225,"Approved")</f>
         <v>0</v>
       </c>
       <c r="J6" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$212,$A6,Items!$G$2:$G$212,"Pending")</f>
+        <f>COUNTIFS(Items!$B$2:$B$225,$A6,Items!$G$2:$G$225,"Pending")</f>
         <v>9</v>
       </c>
       <c r="K6" s="4">
@@ -318,39 +318,39 @@
         </is>
       </c>
       <c r="B7" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$212,$A7)</f>
+        <f>COUNTIFS(Items!$B$2:$B$225,$A7)</f>
         <v>10</v>
       </c>
       <c r="C7" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$212,$A7,Items!$F$2:$F$212,C$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$225,$A7,Items!$F$2:$F$225,C$5)</f>
         <v>10</v>
       </c>
       <c r="D7" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$212,$A7,Items!$F$2:$F$212,D$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$225,$A7,Items!$F$2:$F$225,D$5)</f>
         <v>0</v>
       </c>
       <c r="E7" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$212,$A7,Items!$F$2:$F$212,E$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$225,$A7,Items!$F$2:$F$225,E$5)</f>
         <v>0</v>
       </c>
       <c r="F7" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$212,$A7,Items!$F$2:$F$212,F$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$225,$A7,Items!$F$2:$F$225,F$5)</f>
         <v>0</v>
       </c>
       <c r="G7" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$212,$A7,Items!$F$2:$F$212,G$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$225,$A7,Items!$F$2:$F$225,G$5)</f>
         <v>0</v>
       </c>
       <c r="H7" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$212,$A7,Items!$F$2:$F$212,H$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$225,$A7,Items!$F$2:$F$225,H$5)</f>
         <v>0</v>
       </c>
       <c r="I7" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$212,$A7,Items!$G$2:$G$212,"Approved")</f>
+        <f>COUNTIFS(Items!$B$2:$B$225,$A7,Items!$G$2:$G$225,"Approved")</f>
         <v>0</v>
       </c>
       <c r="J7" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$212,$A7,Items!$G$2:$G$212,"Pending")</f>
+        <f>COUNTIFS(Items!$B$2:$B$225,$A7,Items!$G$2:$G$225,"Pending")</f>
         <v>10</v>
       </c>
       <c r="K7" s="4">
@@ -369,39 +369,39 @@
         </is>
       </c>
       <c r="B8" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$212,$A8)</f>
+        <f>COUNTIFS(Items!$B$2:$B$225,$A8)</f>
         <v>9</v>
       </c>
       <c r="C8" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$212,$A8,Items!$F$2:$F$212,C$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$225,$A8,Items!$F$2:$F$225,C$5)</f>
         <v>8</v>
       </c>
       <c r="D8" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$212,$A8,Items!$F$2:$F$212,D$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$225,$A8,Items!$F$2:$F$225,D$5)</f>
         <v>0</v>
       </c>
       <c r="E8" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$212,$A8,Items!$F$2:$F$212,E$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$225,$A8,Items!$F$2:$F$225,E$5)</f>
         <v>0</v>
       </c>
       <c r="F8" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$212,$A8,Items!$F$2:$F$212,F$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$225,$A8,Items!$F$2:$F$225,F$5)</f>
         <v>1</v>
       </c>
       <c r="G8" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$212,$A8,Items!$F$2:$F$212,G$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$225,$A8,Items!$F$2:$F$225,G$5)</f>
         <v>0</v>
       </c>
       <c r="H8" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$212,$A8,Items!$F$2:$F$212,H$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$225,$A8,Items!$F$2:$F$225,H$5)</f>
         <v>0</v>
       </c>
       <c r="I8" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$212,$A8,Items!$G$2:$G$212,"Approved")</f>
+        <f>COUNTIFS(Items!$B$2:$B$225,$A8,Items!$G$2:$G$225,"Approved")</f>
         <v>0</v>
       </c>
       <c r="J8" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$212,$A8,Items!$G$2:$G$212,"Pending")</f>
+        <f>COUNTIFS(Items!$B$2:$B$225,$A8,Items!$G$2:$G$225,"Pending")</f>
         <v>9</v>
       </c>
       <c r="K8" s="4">
@@ -420,39 +420,39 @@
         </is>
       </c>
       <c r="B9" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$212,$A9)</f>
+        <f>COUNTIFS(Items!$B$2:$B$225,$A9)</f>
         <v>9</v>
       </c>
       <c r="C9" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$212,$A9,Items!$F$2:$F$212,C$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$225,$A9,Items!$F$2:$F$225,C$5)</f>
         <v>9</v>
       </c>
       <c r="D9" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$212,$A9,Items!$F$2:$F$212,D$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$225,$A9,Items!$F$2:$F$225,D$5)</f>
         <v>0</v>
       </c>
       <c r="E9" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$212,$A9,Items!$F$2:$F$212,E$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$225,$A9,Items!$F$2:$F$225,E$5)</f>
         <v>0</v>
       </c>
       <c r="F9" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$212,$A9,Items!$F$2:$F$212,F$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$225,$A9,Items!$F$2:$F$225,F$5)</f>
         <v>0</v>
       </c>
       <c r="G9" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$212,$A9,Items!$F$2:$F$212,G$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$225,$A9,Items!$F$2:$F$225,G$5)</f>
         <v>0</v>
       </c>
       <c r="H9" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$212,$A9,Items!$F$2:$F$212,H$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$225,$A9,Items!$F$2:$F$225,H$5)</f>
         <v>0</v>
       </c>
       <c r="I9" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$212,$A9,Items!$G$2:$G$212,"Approved")</f>
+        <f>COUNTIFS(Items!$B$2:$B$225,$A9,Items!$G$2:$G$225,"Approved")</f>
         <v>0</v>
       </c>
       <c r="J9" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$212,$A9,Items!$G$2:$G$212,"Pending")</f>
+        <f>COUNTIFS(Items!$B$2:$B$225,$A9,Items!$G$2:$G$225,"Pending")</f>
         <v>9</v>
       </c>
       <c r="K9" s="4">
@@ -471,39 +471,39 @@
         </is>
       </c>
       <c r="B10" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$212,$A10)</f>
+        <f>COUNTIFS(Items!$B$2:$B$225,$A10)</f>
         <v>9</v>
       </c>
       <c r="C10" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$212,$A10,Items!$F$2:$F$212,C$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$225,$A10,Items!$F$2:$F$225,C$5)</f>
         <v>9</v>
       </c>
       <c r="D10" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$212,$A10,Items!$F$2:$F$212,D$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$225,$A10,Items!$F$2:$F$225,D$5)</f>
         <v>0</v>
       </c>
       <c r="E10" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$212,$A10,Items!$F$2:$F$212,E$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$225,$A10,Items!$F$2:$F$225,E$5)</f>
         <v>0</v>
       </c>
       <c r="F10" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$212,$A10,Items!$F$2:$F$212,F$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$225,$A10,Items!$F$2:$F$225,F$5)</f>
         <v>0</v>
       </c>
       <c r="G10" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$212,$A10,Items!$F$2:$F$212,G$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$225,$A10,Items!$F$2:$F$225,G$5)</f>
         <v>0</v>
       </c>
       <c r="H10" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$212,$A10,Items!$F$2:$F$212,H$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$225,$A10,Items!$F$2:$F$225,H$5)</f>
         <v>0</v>
       </c>
       <c r="I10" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$212,$A10,Items!$G$2:$G$212,"Approved")</f>
+        <f>COUNTIFS(Items!$B$2:$B$225,$A10,Items!$G$2:$G$225,"Approved")</f>
         <v>0</v>
       </c>
       <c r="J10" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$212,$A10,Items!$G$2:$G$212,"Pending")</f>
+        <f>COUNTIFS(Items!$B$2:$B$225,$A10,Items!$G$2:$G$225,"Pending")</f>
         <v>9</v>
       </c>
       <c r="K10" s="4">
@@ -522,39 +522,39 @@
         </is>
       </c>
       <c r="B11" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$212,$A11)</f>
+        <f>COUNTIFS(Items!$B$2:$B$225,$A11)</f>
         <v>5</v>
       </c>
       <c r="C11" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$212,$A11,Items!$F$2:$F$212,C$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$225,$A11,Items!$F$2:$F$225,C$5)</f>
         <v>5</v>
       </c>
       <c r="D11" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$212,$A11,Items!$F$2:$F$212,D$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$225,$A11,Items!$F$2:$F$225,D$5)</f>
         <v>0</v>
       </c>
       <c r="E11" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$212,$A11,Items!$F$2:$F$212,E$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$225,$A11,Items!$F$2:$F$225,E$5)</f>
         <v>0</v>
       </c>
       <c r="F11" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$212,$A11,Items!$F$2:$F$212,F$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$225,$A11,Items!$F$2:$F$225,F$5)</f>
         <v>0</v>
       </c>
       <c r="G11" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$212,$A11,Items!$F$2:$F$212,G$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$225,$A11,Items!$F$2:$F$225,G$5)</f>
         <v>0</v>
       </c>
       <c r="H11" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$212,$A11,Items!$F$2:$F$212,H$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$225,$A11,Items!$F$2:$F$225,H$5)</f>
         <v>0</v>
       </c>
       <c r="I11" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$212,$A11,Items!$G$2:$G$212,"Approved")</f>
+        <f>COUNTIFS(Items!$B$2:$B$225,$A11,Items!$G$2:$G$225,"Approved")</f>
         <v>0</v>
       </c>
       <c r="J11" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$212,$A11,Items!$G$2:$G$212,"Pending")</f>
+        <f>COUNTIFS(Items!$B$2:$B$225,$A11,Items!$G$2:$G$225,"Pending")</f>
         <v>5</v>
       </c>
       <c r="K11" s="4">
@@ -573,39 +573,39 @@
         </is>
       </c>
       <c r="B12" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$212,$A12)</f>
+        <f>COUNTIFS(Items!$B$2:$B$225,$A12)</f>
         <v>5</v>
       </c>
       <c r="C12" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$212,$A12,Items!$F$2:$F$212,C$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$225,$A12,Items!$F$2:$F$225,C$5)</f>
         <v>5</v>
       </c>
       <c r="D12" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$212,$A12,Items!$F$2:$F$212,D$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$225,$A12,Items!$F$2:$F$225,D$5)</f>
         <v>0</v>
       </c>
       <c r="E12" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$212,$A12,Items!$F$2:$F$212,E$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$225,$A12,Items!$F$2:$F$225,E$5)</f>
         <v>0</v>
       </c>
       <c r="F12" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$212,$A12,Items!$F$2:$F$212,F$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$225,$A12,Items!$F$2:$F$225,F$5)</f>
         <v>0</v>
       </c>
       <c r="G12" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$212,$A12,Items!$F$2:$F$212,G$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$225,$A12,Items!$F$2:$F$225,G$5)</f>
         <v>0</v>
       </c>
       <c r="H12" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$212,$A12,Items!$F$2:$F$212,H$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$225,$A12,Items!$F$2:$F$225,H$5)</f>
         <v>0</v>
       </c>
       <c r="I12" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$212,$A12,Items!$G$2:$G$212,"Approved")</f>
+        <f>COUNTIFS(Items!$B$2:$B$225,$A12,Items!$G$2:$G$225,"Approved")</f>
         <v>0</v>
       </c>
       <c r="J12" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$212,$A12,Items!$G$2:$G$212,"Pending")</f>
+        <f>COUNTIFS(Items!$B$2:$B$225,$A12,Items!$G$2:$G$225,"Pending")</f>
         <v>5</v>
       </c>
       <c r="K12" s="4">
@@ -624,39 +624,39 @@
         </is>
       </c>
       <c r="B13" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$212,$A13)</f>
+        <f>COUNTIFS(Items!$B$2:$B$225,$A13)</f>
         <v>9</v>
       </c>
       <c r="C13" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$212,$A13,Items!$F$2:$F$212,C$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$225,$A13,Items!$F$2:$F$225,C$5)</f>
         <v>9</v>
       </c>
       <c r="D13" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$212,$A13,Items!$F$2:$F$212,D$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$225,$A13,Items!$F$2:$F$225,D$5)</f>
         <v>0</v>
       </c>
       <c r="E13" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$212,$A13,Items!$F$2:$F$212,E$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$225,$A13,Items!$F$2:$F$225,E$5)</f>
         <v>0</v>
       </c>
       <c r="F13" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$212,$A13,Items!$F$2:$F$212,F$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$225,$A13,Items!$F$2:$F$225,F$5)</f>
         <v>0</v>
       </c>
       <c r="G13" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$212,$A13,Items!$F$2:$F$212,G$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$225,$A13,Items!$F$2:$F$225,G$5)</f>
         <v>0</v>
       </c>
       <c r="H13" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$212,$A13,Items!$F$2:$F$212,H$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$225,$A13,Items!$F$2:$F$225,H$5)</f>
         <v>0</v>
       </c>
       <c r="I13" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$212,$A13,Items!$G$2:$G$212,"Approved")</f>
+        <f>COUNTIFS(Items!$B$2:$B$225,$A13,Items!$G$2:$G$225,"Approved")</f>
         <v>0</v>
       </c>
       <c r="J13" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$212,$A13,Items!$G$2:$G$212,"Pending")</f>
+        <f>COUNTIFS(Items!$B$2:$B$225,$A13,Items!$G$2:$G$225,"Pending")</f>
         <v>9</v>
       </c>
       <c r="K13" s="4">
@@ -675,39 +675,39 @@
         </is>
       </c>
       <c r="B14" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$212,$A14)</f>
+        <f>COUNTIFS(Items!$B$2:$B$225,$A14)</f>
         <v>17</v>
       </c>
       <c r="C14" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$212,$A14,Items!$F$2:$F$212,C$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$225,$A14,Items!$F$2:$F$225,C$5)</f>
         <v>17</v>
       </c>
       <c r="D14" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$212,$A14,Items!$F$2:$F$212,D$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$225,$A14,Items!$F$2:$F$225,D$5)</f>
         <v>0</v>
       </c>
       <c r="E14" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$212,$A14,Items!$F$2:$F$212,E$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$225,$A14,Items!$F$2:$F$225,E$5)</f>
         <v>0</v>
       </c>
       <c r="F14" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$212,$A14,Items!$F$2:$F$212,F$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$225,$A14,Items!$F$2:$F$225,F$5)</f>
         <v>0</v>
       </c>
       <c r="G14" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$212,$A14,Items!$F$2:$F$212,G$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$225,$A14,Items!$F$2:$F$225,G$5)</f>
         <v>0</v>
       </c>
       <c r="H14" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$212,$A14,Items!$F$2:$F$212,H$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$225,$A14,Items!$F$2:$F$225,H$5)</f>
         <v>0</v>
       </c>
       <c r="I14" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$212,$A14,Items!$G$2:$G$212,"Approved")</f>
+        <f>COUNTIFS(Items!$B$2:$B$225,$A14,Items!$G$2:$G$225,"Approved")</f>
         <v>0</v>
       </c>
       <c r="J14" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$212,$A14,Items!$G$2:$G$212,"Pending")</f>
+        <f>COUNTIFS(Items!$B$2:$B$225,$A14,Items!$G$2:$G$225,"Pending")</f>
         <v>17</v>
       </c>
       <c r="K14" s="4">
@@ -726,39 +726,39 @@
         </is>
       </c>
       <c r="B15" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$212,$A15)</f>
+        <f>COUNTIFS(Items!$B$2:$B$225,$A15)</f>
         <v>4</v>
       </c>
       <c r="C15" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$212,$A15,Items!$F$2:$F$212,C$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$225,$A15,Items!$F$2:$F$225,C$5)</f>
         <v>4</v>
       </c>
       <c r="D15" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$212,$A15,Items!$F$2:$F$212,D$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$225,$A15,Items!$F$2:$F$225,D$5)</f>
         <v>0</v>
       </c>
       <c r="E15" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$212,$A15,Items!$F$2:$F$212,E$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$225,$A15,Items!$F$2:$F$225,E$5)</f>
         <v>0</v>
       </c>
       <c r="F15" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$212,$A15,Items!$F$2:$F$212,F$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$225,$A15,Items!$F$2:$F$225,F$5)</f>
         <v>0</v>
       </c>
       <c r="G15" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$212,$A15,Items!$F$2:$F$212,G$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$225,$A15,Items!$F$2:$F$225,G$5)</f>
         <v>0</v>
       </c>
       <c r="H15" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$212,$A15,Items!$F$2:$F$212,H$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$225,$A15,Items!$F$2:$F$225,H$5)</f>
         <v>0</v>
       </c>
       <c r="I15" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$212,$A15,Items!$G$2:$G$212,"Approved")</f>
+        <f>COUNTIFS(Items!$B$2:$B$225,$A15,Items!$G$2:$G$225,"Approved")</f>
         <v>0</v>
       </c>
       <c r="J15" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$212,$A15,Items!$G$2:$G$212,"Pending")</f>
+        <f>COUNTIFS(Items!$B$2:$B$225,$A15,Items!$G$2:$G$225,"Pending")</f>
         <v>4</v>
       </c>
       <c r="K15" s="4">
@@ -777,39 +777,39 @@
         </is>
       </c>
       <c r="B16" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$212,$A16)</f>
+        <f>COUNTIFS(Items!$B$2:$B$225,$A16)</f>
         <v>9</v>
       </c>
       <c r="C16" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$212,$A16,Items!$F$2:$F$212,C$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$225,$A16,Items!$F$2:$F$225,C$5)</f>
         <v>9</v>
       </c>
       <c r="D16" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$212,$A16,Items!$F$2:$F$212,D$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$225,$A16,Items!$F$2:$F$225,D$5)</f>
         <v>0</v>
       </c>
       <c r="E16" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$212,$A16,Items!$F$2:$F$212,E$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$225,$A16,Items!$F$2:$F$225,E$5)</f>
         <v>0</v>
       </c>
       <c r="F16" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$212,$A16,Items!$F$2:$F$212,F$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$225,$A16,Items!$F$2:$F$225,F$5)</f>
         <v>0</v>
       </c>
       <c r="G16" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$212,$A16,Items!$F$2:$F$212,G$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$225,$A16,Items!$F$2:$F$225,G$5)</f>
         <v>0</v>
       </c>
       <c r="H16" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$212,$A16,Items!$F$2:$F$212,H$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$225,$A16,Items!$F$2:$F$225,H$5)</f>
         <v>0</v>
       </c>
       <c r="I16" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$212,$A16,Items!$G$2:$G$212,"Approved")</f>
+        <f>COUNTIFS(Items!$B$2:$B$225,$A16,Items!$G$2:$G$225,"Approved")</f>
         <v>0</v>
       </c>
       <c r="J16" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$212,$A16,Items!$G$2:$G$212,"Pending")</f>
+        <f>COUNTIFS(Items!$B$2:$B$225,$A16,Items!$G$2:$G$225,"Pending")</f>
         <v>9</v>
       </c>
       <c r="K16" s="4">
@@ -828,39 +828,39 @@
         </is>
       </c>
       <c r="B17" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$212,$A17)</f>
+        <f>COUNTIFS(Items!$B$2:$B$225,$A17)</f>
         <v>15</v>
       </c>
       <c r="C17" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$212,$A17,Items!$F$2:$F$212,C$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$225,$A17,Items!$F$2:$F$225,C$5)</f>
         <v>14</v>
       </c>
       <c r="D17" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$212,$A17,Items!$F$2:$F$212,D$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$225,$A17,Items!$F$2:$F$225,D$5)</f>
         <v>0</v>
       </c>
       <c r="E17" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$212,$A17,Items!$F$2:$F$212,E$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$225,$A17,Items!$F$2:$F$225,E$5)</f>
         <v>0</v>
       </c>
       <c r="F17" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$212,$A17,Items!$F$2:$F$212,F$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$225,$A17,Items!$F$2:$F$225,F$5)</f>
         <v>1</v>
       </c>
       <c r="G17" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$212,$A17,Items!$F$2:$F$212,G$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$225,$A17,Items!$F$2:$F$225,G$5)</f>
         <v>0</v>
       </c>
       <c r="H17" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$212,$A17,Items!$F$2:$F$212,H$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$225,$A17,Items!$F$2:$F$225,H$5)</f>
         <v>0</v>
       </c>
       <c r="I17" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$212,$A17,Items!$G$2:$G$212,"Approved")</f>
+        <f>COUNTIFS(Items!$B$2:$B$225,$A17,Items!$G$2:$G$225,"Approved")</f>
         <v>0</v>
       </c>
       <c r="J17" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$212,$A17,Items!$G$2:$G$212,"Pending")</f>
+        <f>COUNTIFS(Items!$B$2:$B$225,$A17,Items!$G$2:$G$225,"Pending")</f>
         <v>15</v>
       </c>
       <c r="K17" s="4">
@@ -879,39 +879,39 @@
         </is>
       </c>
       <c r="B18" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$212,$A18)</f>
+        <f>COUNTIFS(Items!$B$2:$B$225,$A18)</f>
         <v>10</v>
       </c>
       <c r="C18" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$212,$A18,Items!$F$2:$F$212,C$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$225,$A18,Items!$F$2:$F$225,C$5)</f>
         <v>10</v>
       </c>
       <c r="D18" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$212,$A18,Items!$F$2:$F$212,D$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$225,$A18,Items!$F$2:$F$225,D$5)</f>
         <v>0</v>
       </c>
       <c r="E18" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$212,$A18,Items!$F$2:$F$212,E$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$225,$A18,Items!$F$2:$F$225,E$5)</f>
         <v>0</v>
       </c>
       <c r="F18" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$212,$A18,Items!$F$2:$F$212,F$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$225,$A18,Items!$F$2:$F$225,F$5)</f>
         <v>0</v>
       </c>
       <c r="G18" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$212,$A18,Items!$F$2:$F$212,G$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$225,$A18,Items!$F$2:$F$225,G$5)</f>
         <v>0</v>
       </c>
       <c r="H18" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$212,$A18,Items!$F$2:$F$212,H$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$225,$A18,Items!$F$2:$F$225,H$5)</f>
         <v>0</v>
       </c>
       <c r="I18" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$212,$A18,Items!$G$2:$G$212,"Approved")</f>
+        <f>COUNTIFS(Items!$B$2:$B$225,$A18,Items!$G$2:$G$225,"Approved")</f>
         <v>0</v>
       </c>
       <c r="J18" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$212,$A18,Items!$G$2:$G$212,"Pending")</f>
+        <f>COUNTIFS(Items!$B$2:$B$225,$A18,Items!$G$2:$G$225,"Pending")</f>
         <v>10</v>
       </c>
       <c r="K18" s="4">
@@ -930,39 +930,39 @@
         </is>
       </c>
       <c r="B19" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$212,$A19)</f>
+        <f>COUNTIFS(Items!$B$2:$B$225,$A19)</f>
         <v>7</v>
       </c>
       <c r="C19" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$212,$A19,Items!$F$2:$F$212,C$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$225,$A19,Items!$F$2:$F$225,C$5)</f>
         <v>7</v>
       </c>
       <c r="D19" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$212,$A19,Items!$F$2:$F$212,D$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$225,$A19,Items!$F$2:$F$225,D$5)</f>
         <v>0</v>
       </c>
       <c r="E19" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$212,$A19,Items!$F$2:$F$212,E$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$225,$A19,Items!$F$2:$F$225,E$5)</f>
         <v>0</v>
       </c>
       <c r="F19" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$212,$A19,Items!$F$2:$F$212,F$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$225,$A19,Items!$F$2:$F$225,F$5)</f>
         <v>0</v>
       </c>
       <c r="G19" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$212,$A19,Items!$F$2:$F$212,G$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$225,$A19,Items!$F$2:$F$225,G$5)</f>
         <v>0</v>
       </c>
       <c r="H19" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$212,$A19,Items!$F$2:$F$212,H$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$225,$A19,Items!$F$2:$F$225,H$5)</f>
         <v>0</v>
       </c>
       <c r="I19" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$212,$A19,Items!$G$2:$G$212,"Approved")</f>
+        <f>COUNTIFS(Items!$B$2:$B$225,$A19,Items!$G$2:$G$225,"Approved")</f>
         <v>0</v>
       </c>
       <c r="J19" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$212,$A19,Items!$G$2:$G$212,"Pending")</f>
+        <f>COUNTIFS(Items!$B$2:$B$225,$A19,Items!$G$2:$G$225,"Pending")</f>
         <v>7</v>
       </c>
       <c r="K19" s="4">
@@ -981,39 +981,39 @@
         </is>
       </c>
       <c r="B20" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$212,$A20)</f>
+        <f>COUNTIFS(Items!$B$2:$B$225,$A20)</f>
         <v>23</v>
       </c>
       <c r="C20" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$212,$A20,Items!$F$2:$F$212,C$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$225,$A20,Items!$F$2:$F$225,C$5)</f>
         <v>23</v>
       </c>
       <c r="D20" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$212,$A20,Items!$F$2:$F$212,D$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$225,$A20,Items!$F$2:$F$225,D$5)</f>
         <v>0</v>
       </c>
       <c r="E20" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$212,$A20,Items!$F$2:$F$212,E$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$225,$A20,Items!$F$2:$F$225,E$5)</f>
         <v>0</v>
       </c>
       <c r="F20" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$212,$A20,Items!$F$2:$F$212,F$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$225,$A20,Items!$F$2:$F$225,F$5)</f>
         <v>0</v>
       </c>
       <c r="G20" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$212,$A20,Items!$F$2:$F$212,G$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$225,$A20,Items!$F$2:$F$225,G$5)</f>
         <v>0</v>
       </c>
       <c r="H20" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$212,$A20,Items!$F$2:$F$212,H$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$225,$A20,Items!$F$2:$F$225,H$5)</f>
         <v>0</v>
       </c>
       <c r="I20" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$212,$A20,Items!$G$2:$G$212,"Approved")</f>
+        <f>COUNTIFS(Items!$B$2:$B$225,$A20,Items!$G$2:$G$225,"Approved")</f>
         <v>0</v>
       </c>
       <c r="J20" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$212,$A20,Items!$G$2:$G$212,"Pending")</f>
+        <f>COUNTIFS(Items!$B$2:$B$225,$A20,Items!$G$2:$G$225,"Pending")</f>
         <v>23</v>
       </c>
       <c r="K20" s="4">
@@ -1032,39 +1032,39 @@
         </is>
       </c>
       <c r="B21" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$212,$A21)</f>
+        <f>COUNTIFS(Items!$B$2:$B$225,$A21)</f>
         <v>2</v>
       </c>
       <c r="C21" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$212,$A21,Items!$F$2:$F$212,C$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$225,$A21,Items!$F$2:$F$225,C$5)</f>
         <v>2</v>
       </c>
       <c r="D21" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$212,$A21,Items!$F$2:$F$212,D$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$225,$A21,Items!$F$2:$F$225,D$5)</f>
         <v>0</v>
       </c>
       <c r="E21" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$212,$A21,Items!$F$2:$F$212,E$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$225,$A21,Items!$F$2:$F$225,E$5)</f>
         <v>0</v>
       </c>
       <c r="F21" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$212,$A21,Items!$F$2:$F$212,F$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$225,$A21,Items!$F$2:$F$225,F$5)</f>
         <v>0</v>
       </c>
       <c r="G21" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$212,$A21,Items!$F$2:$F$212,G$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$225,$A21,Items!$F$2:$F$225,G$5)</f>
         <v>0</v>
       </c>
       <c r="H21" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$212,$A21,Items!$F$2:$F$212,H$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$225,$A21,Items!$F$2:$F$225,H$5)</f>
         <v>0</v>
       </c>
       <c r="I21" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$212,$A21,Items!$G$2:$G$212,"Approved")</f>
+        <f>COUNTIFS(Items!$B$2:$B$225,$A21,Items!$G$2:$G$225,"Approved")</f>
         <v>0</v>
       </c>
       <c r="J21" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$212,$A21,Items!$G$2:$G$212,"Pending")</f>
+        <f>COUNTIFS(Items!$B$2:$B$225,$A21,Items!$G$2:$G$225,"Pending")</f>
         <v>2</v>
       </c>
       <c r="K21" s="4">
@@ -1083,39 +1083,39 @@
         </is>
       </c>
       <c r="B22" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$212,$A22)</f>
+        <f>COUNTIFS(Items!$B$2:$B$225,$A22)</f>
         <v>6</v>
       </c>
       <c r="C22" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$212,$A22,Items!$F$2:$F$212,C$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$225,$A22,Items!$F$2:$F$225,C$5)</f>
         <v>6</v>
       </c>
       <c r="D22" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$212,$A22,Items!$F$2:$F$212,D$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$225,$A22,Items!$F$2:$F$225,D$5)</f>
         <v>0</v>
       </c>
       <c r="E22" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$212,$A22,Items!$F$2:$F$212,E$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$225,$A22,Items!$F$2:$F$225,E$5)</f>
         <v>0</v>
       </c>
       <c r="F22" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$212,$A22,Items!$F$2:$F$212,F$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$225,$A22,Items!$F$2:$F$225,F$5)</f>
         <v>0</v>
       </c>
       <c r="G22" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$212,$A22,Items!$F$2:$F$212,G$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$225,$A22,Items!$F$2:$F$225,G$5)</f>
         <v>0</v>
       </c>
       <c r="H22" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$212,$A22,Items!$F$2:$F$212,H$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$225,$A22,Items!$F$2:$F$225,H$5)</f>
         <v>0</v>
       </c>
       <c r="I22" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$212,$A22,Items!$G$2:$G$212,"Approved")</f>
+        <f>COUNTIFS(Items!$B$2:$B$225,$A22,Items!$G$2:$G$225,"Approved")</f>
         <v>0</v>
       </c>
       <c r="J22" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$212,$A22,Items!$G$2:$G$212,"Pending")</f>
+        <f>COUNTIFS(Items!$B$2:$B$225,$A22,Items!$G$2:$G$225,"Pending")</f>
         <v>6</v>
       </c>
       <c r="K22" s="4">
@@ -1134,39 +1134,39 @@
         </is>
       </c>
       <c r="B23" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$212,$A23)</f>
+        <f>COUNTIFS(Items!$B$2:$B$225,$A23)</f>
         <v>23</v>
       </c>
       <c r="C23" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$212,$A23,Items!$F$2:$F$212,C$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$225,$A23,Items!$F$2:$F$225,C$5)</f>
         <v>22</v>
       </c>
       <c r="D23" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$212,$A23,Items!$F$2:$F$212,D$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$225,$A23,Items!$F$2:$F$225,D$5)</f>
         <v>0</v>
       </c>
       <c r="E23" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$212,$A23,Items!$F$2:$F$212,E$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$225,$A23,Items!$F$2:$F$225,E$5)</f>
         <v>0</v>
       </c>
       <c r="F23" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$212,$A23,Items!$F$2:$F$212,F$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$225,$A23,Items!$F$2:$F$225,F$5)</f>
         <v>1</v>
       </c>
       <c r="G23" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$212,$A23,Items!$F$2:$F$212,G$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$225,$A23,Items!$F$2:$F$225,G$5)</f>
         <v>0</v>
       </c>
       <c r="H23" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$212,$A23,Items!$F$2:$F$212,H$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$225,$A23,Items!$F$2:$F$225,H$5)</f>
         <v>0</v>
       </c>
       <c r="I23" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$212,$A23,Items!$G$2:$G$212,"Approved")</f>
+        <f>COUNTIFS(Items!$B$2:$B$225,$A23,Items!$G$2:$G$225,"Approved")</f>
         <v>0</v>
       </c>
       <c r="J23" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$212,$A23,Items!$G$2:$G$212,"Pending")</f>
+        <f>COUNTIFS(Items!$B$2:$B$225,$A23,Items!$G$2:$G$225,"Pending")</f>
         <v>23</v>
       </c>
       <c r="K23" s="4">
@@ -1185,39 +1185,39 @@
         </is>
       </c>
       <c r="B24" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$212,$A24)</f>
+        <f>COUNTIFS(Items!$B$2:$B$225,$A24)</f>
         <v>4</v>
       </c>
       <c r="C24" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$212,$A24,Items!$F$2:$F$212,C$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$225,$A24,Items!$F$2:$F$225,C$5)</f>
         <v>2</v>
       </c>
       <c r="D24" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$212,$A24,Items!$F$2:$F$212,D$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$225,$A24,Items!$F$2:$F$225,D$5)</f>
         <v>0</v>
       </c>
       <c r="E24" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$212,$A24,Items!$F$2:$F$212,E$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$225,$A24,Items!$F$2:$F$225,E$5)</f>
         <v>0</v>
       </c>
       <c r="F24" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$212,$A24,Items!$F$2:$F$212,F$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$225,$A24,Items!$F$2:$F$225,F$5)</f>
         <v>0</v>
       </c>
       <c r="G24" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$212,$A24,Items!$F$2:$F$212,G$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$225,$A24,Items!$F$2:$F$225,G$5)</f>
         <v>2</v>
       </c>
       <c r="H24" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$212,$A24,Items!$F$2:$F$212,H$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$225,$A24,Items!$F$2:$F$225,H$5)</f>
         <v>0</v>
       </c>
       <c r="I24" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$212,$A24,Items!$G$2:$G$212,"Approved")</f>
+        <f>COUNTIFS(Items!$B$2:$B$225,$A24,Items!$G$2:$G$225,"Approved")</f>
         <v>0</v>
       </c>
       <c r="J24" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$212,$A24,Items!$G$2:$G$212,"Pending")</f>
+        <f>COUNTIFS(Items!$B$2:$B$225,$A24,Items!$G$2:$G$225,"Pending")</f>
         <v>4</v>
       </c>
       <c r="K24" s="4">
@@ -1236,40 +1236,40 @@
         </is>
       </c>
       <c r="B25" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$212,$A25)</f>
-        <v>9</v>
+        <f>COUNTIFS(Items!$B$2:$B$225,$A25)</f>
+        <v>22</v>
       </c>
       <c r="C25" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$212,$A25,Items!$F$2:$F$212,C$5)</f>
-        <v>8</v>
+        <f>COUNTIFS(Items!$B$2:$B$225,$A25,Items!$F$2:$F$225,C$5)</f>
+        <v>21</v>
       </c>
       <c r="D25" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$212,$A25,Items!$F$2:$F$212,D$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$225,$A25,Items!$F$2:$F$225,D$5)</f>
         <v>0</v>
       </c>
       <c r="E25" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$212,$A25,Items!$F$2:$F$212,E$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$225,$A25,Items!$F$2:$F$225,E$5)</f>
         <v>0</v>
       </c>
       <c r="F25" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$212,$A25,Items!$F$2:$F$212,F$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$225,$A25,Items!$F$2:$F$225,F$5)</f>
         <v>0</v>
       </c>
       <c r="G25" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$212,$A25,Items!$F$2:$F$212,G$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$225,$A25,Items!$F$2:$F$225,G$5)</f>
         <v>1</v>
       </c>
       <c r="H25" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$212,$A25,Items!$F$2:$F$212,H$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$225,$A25,Items!$F$2:$F$225,H$5)</f>
         <v>0</v>
       </c>
       <c r="I25" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$212,$A25,Items!$G$2:$G$212,"Approved")</f>
+        <f>COUNTIFS(Items!$B$2:$B$225,$A25,Items!$G$2:$G$225,"Approved")</f>
         <v>0</v>
       </c>
       <c r="J25" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$212,$A25,Items!$G$2:$G$212,"Pending")</f>
-        <v>9</v>
+        <f>COUNTIFS(Items!$B$2:$B$225,$A25,Items!$G$2:$G$225,"Pending")</f>
+        <v>22</v>
       </c>
       <c r="K25" s="4">
         <f>IF(B25-G25=0,0,(D25+E25+F25)/(B25-G25))</f>
@@ -1287,39 +1287,39 @@
         </is>
       </c>
       <c r="B26" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$212,$A26)</f>
+        <f>COUNTIFS(Items!$B$2:$B$225,$A26)</f>
         <v>3</v>
       </c>
       <c r="C26" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$212,$A26,Items!$F$2:$F$212,C$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$225,$A26,Items!$F$2:$F$225,C$5)</f>
         <v>3</v>
       </c>
       <c r="D26" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$212,$A26,Items!$F$2:$F$212,D$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$225,$A26,Items!$F$2:$F$225,D$5)</f>
         <v>0</v>
       </c>
       <c r="E26" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$212,$A26,Items!$F$2:$F$212,E$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$225,$A26,Items!$F$2:$F$225,E$5)</f>
         <v>0</v>
       </c>
       <c r="F26" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$212,$A26,Items!$F$2:$F$212,F$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$225,$A26,Items!$F$2:$F$225,F$5)</f>
         <v>0</v>
       </c>
       <c r="G26" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$212,$A26,Items!$F$2:$F$212,G$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$225,$A26,Items!$F$2:$F$225,G$5)</f>
         <v>0</v>
       </c>
       <c r="H26" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$212,$A26,Items!$F$2:$F$212,H$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$225,$A26,Items!$F$2:$F$225,H$5)</f>
         <v>0</v>
       </c>
       <c r="I26" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$212,$A26,Items!$G$2:$G$212,"Approved")</f>
+        <f>COUNTIFS(Items!$B$2:$B$225,$A26,Items!$G$2:$G$225,"Approved")</f>
         <v>0</v>
       </c>
       <c r="J26" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$212,$A26,Items!$G$2:$G$212,"Pending")</f>
+        <f>COUNTIFS(Items!$B$2:$B$225,$A26,Items!$G$2:$G$225,"Pending")</f>
         <v>3</v>
       </c>
       <c r="K26" s="4">
@@ -1338,39 +1338,39 @@
         </is>
       </c>
       <c r="B27" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$212,$A27)</f>
+        <f>COUNTIFS(Items!$B$2:$B$225,$A27)</f>
         <v>14</v>
       </c>
       <c r="C27" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$212,$A27,Items!$F$2:$F$212,C$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$225,$A27,Items!$F$2:$F$225,C$5)</f>
         <v>14</v>
       </c>
       <c r="D27" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$212,$A27,Items!$F$2:$F$212,D$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$225,$A27,Items!$F$2:$F$225,D$5)</f>
         <v>0</v>
       </c>
       <c r="E27" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$212,$A27,Items!$F$2:$F$212,E$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$225,$A27,Items!$F$2:$F$225,E$5)</f>
         <v>0</v>
       </c>
       <c r="F27" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$212,$A27,Items!$F$2:$F$212,F$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$225,$A27,Items!$F$2:$F$225,F$5)</f>
         <v>0</v>
       </c>
       <c r="G27" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$212,$A27,Items!$F$2:$F$212,G$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$225,$A27,Items!$F$2:$F$225,G$5)</f>
         <v>0</v>
       </c>
       <c r="H27" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$212,$A27,Items!$F$2:$F$212,H$5)</f>
+        <f>COUNTIFS(Items!$B$2:$B$225,$A27,Items!$F$2:$F$225,H$5)</f>
         <v>0</v>
       </c>
       <c r="I27" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$212,$A27,Items!$G$2:$G$212,"Approved")</f>
+        <f>COUNTIFS(Items!$B$2:$B$225,$A27,Items!$G$2:$G$225,"Approved")</f>
         <v>0</v>
       </c>
       <c r="J27" s="0">
-        <f>COUNTIFS(Items!$B$2:$B$212,$A27,Items!$G$2:$G$212,"Pending")</f>
+        <f>COUNTIFS(Items!$B$2:$B$225,$A27,Items!$G$2:$G$225,"Pending")</f>
         <v>14</v>
       </c>
       <c r="K27" s="4">
@@ -1390,11 +1390,11 @@
       </c>
       <c r="B28" s="5">
         <f>SUM(B6:B27)</f>
-        <v>211</v>
+        <v>224</v>
       </c>
       <c r="C28" s="5">
         <f>SUM(C6:C27)</f>
-        <v>205</v>
+        <v>218</v>
       </c>
       <c r="D28" s="5">
         <f>SUM(D6:D27)</f>
@@ -1422,11 +1422,11 @@
       </c>
       <c r="J28" s="5">
         <f>SUM(J6:J27)</f>
-        <v>211</v>
+        <v>224</v>
       </c>
       <c r="K28" s="4">
         <f>IF(B28-G28=0,0,(D28+E28+F28)/(B28-G28))</f>
-        <v>0.014218</v>
+        <v>0.013393</v>
       </c>
       <c r="L28" s="4">
         <f>IF(B28-G28=0,0,H28/(B28-G28))</f>
@@ -1452,7 +1452,7 @@
         </is>
       </c>
       <c r="B31" s="0">
-        <f>COUNTIFS(Items!$F$2:$F$212,"Failed")</f>
+        <f>COUNTIFS(Items!$F$2:$F$225,"Failed")</f>
         <v>0</v>
       </c>
     </row>
@@ -1463,7 +1463,7 @@
         </is>
       </c>
       <c r="B32" s="0">
-        <f>COUNTIFS(Items!$F$2:$F$212,"Needs improvement")</f>
+        <f>COUNTIFS(Items!$F$2:$F$225,"Needs improvement")</f>
         <v>3</v>
       </c>
     </row>
@@ -1474,7 +1474,7 @@
         </is>
       </c>
       <c r="B33" s="0">
-        <f>COUNTIFS(Items!$F$2:$F$212,"Blocked")</f>
+        <f>COUNTIFS(Items!$F$2:$F$225,"Blocked")</f>
         <v>3</v>
       </c>
     </row>
@@ -1485,7 +1485,7 @@
         </is>
       </c>
       <c r="B34" s="0">
-        <f>COUNTIFS(Items!$L$2:$L$212,"&lt;&gt;",Items!$F$2:$F$212,"&lt;&gt;Passed")</f>
+        <f>COUNTIFS(Items!$L$2:$L$225,"&lt;&gt;",Items!$F$2:$F$225,"&lt;&gt;Passed")</f>
         <v>11</v>
       </c>
     </row>
@@ -1496,8 +1496,8 @@
         </is>
       </c>
       <c r="B35" s="0">
-        <f>COUNTIFS(Items!$H$2:$H$212,"&lt;&gt;")</f>
-        <v>71</v>
+        <f>COUNTIFS(Items!$H$2:$H$225,"&lt;&gt;")</f>
+        <v>83</v>
       </c>
     </row>
   </sheetData>
@@ -22087,6 +22087,1267 @@
         </is>
       </c>
       <c r="S212" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CICD-01</t>
+        </is>
+      </c>
+      <c r="B213" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Server and Deployment</t>
+        </is>
+      </c>
+      <c r="C213" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Actions › Windows packaging › Upload path confinement</t>
+        </is>
+      </c>
+      <c r="D213" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Windows package jobs pass test_server: staged uploads are judged on canonical paths, an alias or 8.3 short data directory works, traversal, symlink escape and invalid names are still refused.</t>
+        </is>
+      </c>
+      <c r="E213" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Critical</t>
+        </is>
+      </c>
+      <c r="F213" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not tested</t>
+        </is>
+      </c>
+      <c r="G213" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pending</t>
+        </is>
+      </c>
+      <c r="H213" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">backend/tests/test_server.py (UploadPathTests)</t>
+        </is>
+      </c>
+      <c r="I213" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="J213" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="K213" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="L213" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="M213" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="N213" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Re-run a Windows package build on GitHub after approval and confirm test_server passes on the runner.</t>
+        </is>
+      </c>
+      <c r="O213" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fixed the test fixture, not the application: confinement is unchanged. Reproduced on Linux with an alias directory. Not run on a Windows runner since the fix.</t>
+        </is>
+      </c>
+      <c r="P213" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">docs/deployment/BUILD.md; backend/server.py; backend/tests/test_server.py</t>
+        </is>
+      </c>
+      <c r="Q213" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Implemented</t>
+        </is>
+      </c>
+      <c r="R213" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Unclassified</t>
+        </is>
+      </c>
+      <c r="S213" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CICD-02</t>
+        </is>
+      </c>
+      <c r="B214" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Server and Deployment</t>
+        </is>
+      </c>
+      <c r="C214" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Actions › Fast Validation › Change-based selection</t>
+        </is>
+      </c>
+      <c r="D214" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pushes to work/main and PRs to main run cheap checks chosen from the change: documentation-only skips Node, frontend changes add build/lint/smoke, backend or unmapped paths run the whole backend; no complete browser suite per push.</t>
+        </is>
+      </c>
+      <c r="E214" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">High</t>
+        </is>
+      </c>
+      <c r="F214" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not tested</t>
+        </is>
+      </c>
+      <c r="G214" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pending</t>
+        </is>
+      </c>
+      <c r="H214" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">backend/tests/test_test_profiles.py (ChangeSelectionTests); backend/tests/test_workflows.py</t>
+        </is>
+      </c>
+      <c r="I214" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="J214" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="K214" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="L214" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="M214" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="N214" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Observe a documentation-only push, a frontend push and a pull request.</t>
+        </is>
+      </c>
+      <c r="O214" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Backend-only selection ran on GitHub in about 1.5 minutes (run 41335937097). Frontend and PR paths are verified offline only.</t>
+        </is>
+      </c>
+      <c r="P214" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">docs/deployment/CI_CD.md; .github/workflows/validate.yml; scripts/test-map.json; scripts/run-tests.py</t>
+        </is>
+      </c>
+      <c r="Q214" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Implemented</t>
+        </is>
+      </c>
+      <c r="R214" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Unclassified</t>
+        </is>
+      </c>
+      <c r="S214" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CICD-03</t>
+        </is>
+      </c>
+      <c r="B215" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Server and Deployment</t>
+        </is>
+      </c>
+      <c r="C215" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Actions › Full Validation › Manual regression</t>
+        </is>
+      </c>
+      <c r="D215" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Full Validation runs only by manual dispatch, runs the complete backend and browser suites, uploads reports, and no other workflow or publication step depends on it.</t>
+        </is>
+      </c>
+      <c r="E215" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">High</t>
+        </is>
+      </c>
+      <c r="F215" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not tested</t>
+        </is>
+      </c>
+      <c r="G215" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pending</t>
+        </is>
+      </c>
+      <c r="H215" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">backend/tests/test_workflows.py</t>
+        </is>
+      </c>
+      <c r="I215" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="J215" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="K215" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="L215" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="M215" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="N215" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">After approval, dispatch once and check both jobs and the uploaded reports.</t>
+        </is>
+      </c>
+      <c r="O215" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The manual form has not run on GitHub.</t>
+        </is>
+      </c>
+      <c r="P215" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">docs/deployment/CI_CD.md; .github/workflows/full-validation.yml</t>
+        </is>
+      </c>
+      <c r="Q215" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Implemented</t>
+        </is>
+      </c>
+      <c r="R215" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Unclassified</t>
+        </is>
+      </c>
+      <c r="S215" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CICD-04</t>
+        </is>
+      </c>
+      <c r="B216" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Server and Deployment</t>
+        </is>
+      </c>
+      <c r="C216" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Actions › Build &amp; Release › No regression prerequisite</t>
+        </is>
+      </c>
+      <c r="D216" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Build Deployment Packages and the legacy Windows build run only lightweight checks; no complete backend or browser suite, status check, approval input or receipt entry requires a prior Full Regression.</t>
+        </is>
+      </c>
+      <c r="E216" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Critical</t>
+        </is>
+      </c>
+      <c r="F216" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not tested</t>
+        </is>
+      </c>
+      <c r="G216" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pending</t>
+        </is>
+      </c>
+      <c r="H216" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">backend/tests/test_workflows.py; backend/tests/test_deployment_packaging.py; backend/tests/test_release_automation.py</t>
+        </is>
+      </c>
+      <c r="I216" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="J216" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="K216" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="L216" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="M216" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="N216" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">After approval, dispatch a build-only run and confirm shared validation completes in minutes without the suites.</t>
+        </is>
+      </c>
+      <c r="O216" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Baseline run 41331855340 spent about 23 of 24.7 minutes in the shared validation suites; they were removed from the release path. Runtime effect (minutes saved) is not measured on GitHub yet.</t>
+        </is>
+      </c>
+      <c r="P216" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">docs/deployment/CI_CD.md; .github/workflows/build-deployments.yml; scripts/deployment-package.py</t>
+        </is>
+      </c>
+      <c r="Q216" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Implemented</t>
+        </is>
+      </c>
+      <c r="R216" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Unclassified</t>
+        </is>
+      </c>
+      <c r="S216" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CICD-05</t>
+        </is>
+      </c>
+      <c r="B217" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Server and Deployment</t>
+        </is>
+      </c>
+      <c r="C217" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Actions › Windows Desktop package</t>
+        </is>
+      </c>
+      <c r="D217" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The windows-desktop target builds, passes the native smoke test and distribution round trip, and uploads a verified archive.</t>
+        </is>
+      </c>
+      <c r="E217" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">High</t>
+        </is>
+      </c>
+      <c r="F217" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not tested</t>
+        </is>
+      </c>
+      <c r="G217" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pending</t>
+        </is>
+      </c>
+      <c r="H217" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">backend/tests/test_deployment_packaging.py; backend/tests/test_windows_package.py</t>
+        </is>
+      </c>
+      <c r="I217" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="J217" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="K217" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="L217" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="M217" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="N217" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Dispatch windows-desktop after approval and check the artifact and the smoke test.</t>
+        </is>
+      </c>
+      <c r="O217" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Needs a Windows runner; failed before the CICD-01 fix and has not been rerun.</t>
+        </is>
+      </c>
+      <c r="P217" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">docs/deployment/WINDOWS_DESKTOP.md; docs/validation/WORKFLOW_MATRIX.md</t>
+        </is>
+      </c>
+      <c r="Q217" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Implemented</t>
+        </is>
+      </c>
+      <c r="R217" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Unclassified</t>
+        </is>
+      </c>
+      <c r="S217" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CICD-06</t>
+        </is>
+      </c>
+      <c r="B218" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Server and Deployment</t>
+        </is>
+      </c>
+      <c r="C218" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Actions › Windows Service package</t>
+        </is>
+      </c>
+      <c r="D218" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The windows-service target builds, verifies the WinSW/SCM package contents and round trip, and uploads a verified archive.</t>
+        </is>
+      </c>
+      <c r="E218" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">High</t>
+        </is>
+      </c>
+      <c r="F218" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not tested</t>
+        </is>
+      </c>
+      <c r="G218" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pending</t>
+        </is>
+      </c>
+      <c r="H218" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">backend/tests/test_deployment_packaging.py</t>
+        </is>
+      </c>
+      <c r="I218" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="J218" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="K218" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="L218" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="M218" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="N218" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Dispatch windows-service after approval; install on a test host to confirm SCM behavior.</t>
+        </is>
+      </c>
+      <c r="O218" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Needs a Windows runner and a real SCM host; not run.</t>
+        </is>
+      </c>
+      <c r="P218" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">docs/deployment/WINDOWS_SERVICE.md; docs/validation/WORKFLOW_MATRIX.md</t>
+        </is>
+      </c>
+      <c r="Q218" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Implemented</t>
+        </is>
+      </c>
+      <c r="R218" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Unclassified</t>
+        </is>
+      </c>
+      <c r="S218" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CICD-07</t>
+        </is>
+      </c>
+      <c r="B219" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Server and Deployment</t>
+        </is>
+      </c>
+      <c r="C219" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Actions › Linux Docker package</t>
+        </is>
+      </c>
+      <c r="D219" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The linux-docker target builds the image archive, passes the container smoke test and round trip.</t>
+        </is>
+      </c>
+      <c r="E219" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">High</t>
+        </is>
+      </c>
+      <c r="F219" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not tested</t>
+        </is>
+      </c>
+      <c r="G219" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pending</t>
+        </is>
+      </c>
+      <c r="H219" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">backend/tests/test_deployment_packaging.py; backend/tests/test_deployment_contracts.py</t>
+        </is>
+      </c>
+      <c r="I219" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="J219" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="K219" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="L219" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="M219" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="N219" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Dispatch linux-docker after approval; run the image on a test host.</t>
+        </is>
+      </c>
+      <c r="O219" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Docker was not run locally; no GitHub run since the change.</t>
+        </is>
+      </c>
+      <c r="P219" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">docs/deployment/LINUX_DOCKER.md; docs/validation/WORKFLOW_MATRIX.md</t>
+        </is>
+      </c>
+      <c r="Q219" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Implemented</t>
+        </is>
+      </c>
+      <c r="R219" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Unclassified</t>
+        </is>
+      </c>
+      <c r="S219" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CICD-08</t>
+        </is>
+      </c>
+      <c r="B220" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Server and Deployment</t>
+        </is>
+      </c>
+      <c r="C220" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Actions › Linux Native package</t>
+        </is>
+      </c>
+      <c r="D220" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The linux-native target builds the archive, validates the systemd unit and round trip.</t>
+        </is>
+      </c>
+      <c r="E220" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">High</t>
+        </is>
+      </c>
+      <c r="F220" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not tested</t>
+        </is>
+      </c>
+      <c r="G220" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pending</t>
+        </is>
+      </c>
+      <c r="H220" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">backend/tests/test_deployment_packaging.py; backend/tests/test_deployment_contracts.py</t>
+        </is>
+      </c>
+      <c r="I220" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="J220" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="K220" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="L220" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="M220" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="N220" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Dispatch linux-native after approval; install on a host with systemd.</t>
+        </is>
+      </c>
+      <c r="O220" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Real systemd was not booted; no GitHub run since the change.</t>
+        </is>
+      </c>
+      <c r="P220" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">docs/deployment/LINUX_NATIVE.md; docs/validation/WORKFLOW_MATRIX.md</t>
+        </is>
+      </c>
+      <c r="Q220" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Implemented</t>
+        </is>
+      </c>
+      <c r="R220" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Unclassified</t>
+        </is>
+      </c>
+      <c r="S220" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CICD-09</t>
+        </is>
+      </c>
+      <c r="B221" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Server and Deployment</t>
+        </is>
+      </c>
+      <c r="C221" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Actions › Release channels and versions</t>
+        </is>
+      </c>
+      <c r="D221" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Alpha, Beta, Release Candidate and Stable produce the expected versions and tags; invalid versions or sequences are rejected; Stable is published only from main; duplicate versions are refused.</t>
+        </is>
+      </c>
+      <c r="E221" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">High</t>
+        </is>
+      </c>
+      <c r="F221" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not tested</t>
+        </is>
+      </c>
+      <c r="G221" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pending</t>
+        </is>
+      </c>
+      <c r="H221" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">backend/tests/test_deployment_release.py</t>
+        </is>
+      </c>
+      <c r="I221" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="J221" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="K221" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="L221" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="M221" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="N221" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">After approval, publish one Beta test release and check tag, flags and assets.</t>
+        </is>
+      </c>
+      <c r="O221" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Stable-from-main is enforced in code (plan job and publish). No test release has been published; publication is verified against a fake API only.</t>
+        </is>
+      </c>
+      <c r="P221" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">docs/deployment/RELEASES.md; docs/validation/WORKFLOW_MATRIX.md</t>
+        </is>
+      </c>
+      <c r="Q221" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Implemented</t>
+        </is>
+      </c>
+      <c r="R221" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Unclassified</t>
+        </is>
+      </c>
+      <c r="S221" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CICD-10</t>
+        </is>
+      </c>
+      <c r="B222" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Server and Deployment</t>
+        </is>
+      </c>
+      <c r="C222" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Actions › Artifact verification and provenance</t>
+        </is>
+      </c>
+      <c r="D222" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Only same-run, same-commit artifacts of selected packages are collected; digests and checksums are verified; a missing, corrupted or unselected artifact stops publication before any release exists.</t>
+        </is>
+      </c>
+      <c r="E222" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Critical</t>
+        </is>
+      </c>
+      <c r="F222" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not tested</t>
+        </is>
+      </c>
+      <c r="G222" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pending</t>
+        </is>
+      </c>
+      <c r="H222" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">backend/tests/test_deployment_release.py; backend/tests/test_deployment_packaging.py</t>
+        </is>
+      </c>
+      <c r="I222" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="J222" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="K222" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="L222" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="M222" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="N222" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Review a real run: artifact IDs, digests and the sealed receipt.</t>
+        </is>
+      </c>
+      <c r="O222" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Offline only; no real publication run.</t>
+        </is>
+      </c>
+      <c r="P222" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">docs/deployment/CI_CD.md; docs/validation/WORKFLOW_MATRIX.md</t>
+        </is>
+      </c>
+      <c r="Q222" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Implemented</t>
+        </is>
+      </c>
+      <c r="R222" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Unclassified</t>
+        </is>
+      </c>
+      <c r="S222" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CICD-11</t>
+        </is>
+      </c>
+      <c r="B223" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Server and Deployment</t>
+        </is>
+      </c>
+      <c r="C223" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Actions › Workflow execution contracts</t>
+        </is>
+      </c>
+      <c r="D223" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The offline contract (triggers, permissions, graph, conditions, policy) fails on any drift, and actionlint passes.</t>
+        </is>
+      </c>
+      <c r="E223" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">High</t>
+        </is>
+      </c>
+      <c r="F223" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not tested</t>
+        </is>
+      </c>
+      <c r="G223" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pending</t>
+        </is>
+      </c>
+      <c r="H223" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">backend/tests/test_workflows.py; backend/tests/test_deployment_selection.py</t>
+        </is>
+      </c>
+      <c r="I223" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="J223" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="K223" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="L223" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="M223" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="N223" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Run python scripts/check-workflows.py after editing any workflow.</t>
+        </is>
+      </c>
+      <c r="O223" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Contracts and actionlint passed on GitHub in run 41335937097. Contracts check structure, not runner behavior.</t>
+        </is>
+      </c>
+      <c r="P223" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">scripts/check-workflows.py; docs/deployment/CI_CD.md</t>
+        </is>
+      </c>
+      <c r="Q223" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Implemented</t>
+        </is>
+      </c>
+      <c r="R223" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Unclassified</t>
+        </is>
+      </c>
+      <c r="S223" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CICD-12</t>
+        </is>
+      </c>
+      <c r="B224" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Server and Deployment</t>
+        </is>
+      </c>
+      <c r="C224" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Actions › CI/CD security</t>
+        </is>
+      </c>
+      <c r="D224" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Actions are SHA-pinned, checkout does not persist credentials, no pull_request_target, least-privilege tokens, inputs only via env, publication gated by channel environments.</t>
+        </is>
+      </c>
+      <c r="E224" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">High</t>
+        </is>
+      </c>
+      <c r="F224" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not tested</t>
+        </is>
+      </c>
+      <c r="G224" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pending</t>
+        </is>
+      </c>
+      <c r="H224" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">backend/tests/test_workflows.py; backend/tests/test_deployment_release.py</t>
+        </is>
+      </c>
+      <c r="I224" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="J224" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="K224" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="L224" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="M224" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="N224" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Confirm environment protection rules (required reviewers, main-only for sap-lens-stable) in repository settings.</t>
+        </is>
+      </c>
+      <c r="O224" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Repository audit: no confirmed issue left open; Stable-from-main gap fixed. Hardening recommendations are listed in the guide. Repository and environment settings cannot be read from the repository.</t>
+        </is>
+      </c>
+      <c r="P224" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">docs/deployment/CI_CD.md; docs/deployment/RELEASES.md</t>
+        </is>
+      </c>
+      <c r="Q224" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Implemented</t>
+        </is>
+      </c>
+      <c r="R224" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Unclassified</t>
+        </is>
+      </c>
+      <c r="S224" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not started</t>
+        </is>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CICD-13</t>
+        </is>
+      </c>
+      <c r="B225" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Server and Deployment</t>
+        </is>
+      </c>
+      <c r="C225" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Actions › GitHub runtime validation</t>
+        </is>
+      </c>
+      <c r="D225" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Each workflow scenario in the matrix is verified by a completed GitHub run recorded with its URL.</t>
+        </is>
+      </c>
+      <c r="E225" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">High</t>
+        </is>
+      </c>
+      <c r="F225" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not tested</t>
+        </is>
+      </c>
+      <c r="G225" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pending</t>
+        </is>
+      </c>
+      <c r="H225" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="I225" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="J225" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="K225" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="L225" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="M225" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="N225" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">After approval, run the smallest set listed in the matrix: Windows package, Linux package, build-only, skipped jobs, safe publication.</t>
+        </is>
+      </c>
+      <c r="O225" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fast Validation backend-only path verified (run 41335937097); the rest is pending. No workflow has been dispatched and no test release published without approval.</t>
+        </is>
+      </c>
+      <c r="P225" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">docs/validation/WORKFLOW_MATRIX.md</t>
+        </is>
+      </c>
+      <c r="Q225" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Partially implemented</t>
+        </is>
+      </c>
+      <c r="R225" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Unclassified</t>
+        </is>
+      </c>
+      <c r="S225" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Not started</t>
         </is>

</xml_diff>

<commit_message>
docs(packaging): record deployment repairs and targeted acceptance evidence
</commit_message>
<xml_diff>
--- a/docs/validation/validation-tracker.xlsx
+++ b/docs/validation/validation-tracker.xlsx
@@ -1497,7 +1497,7 @@
       </c>
       <c r="B35" s="0">
         <f>COUNTIFS(Items!$H$2:$H$225,"&lt;&gt;")</f>
-        <v>83</v>
+        <v>84</v>
       </c>
     </row>
   </sheetData>
@@ -22518,7 +22518,7 @@
       </c>
       <c r="H217" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">backend/tests/test_deployment_packaging.py; backend/tests/test_windows_package.py</t>
+          <t xml:space="preserve">backend/tests/test_windows_package.py; backend/tests/test_deployment_packaging.py</t>
         </is>
       </c>
       <c r="I217" s="2" t="inlineStr">
@@ -22533,7 +22533,7 @@
       </c>
       <c r="K217" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Run 41340859408 (2026-11-01): Desktop failed during build identity verification: the job omitted SAP_LENS_EXPECTED_BUILD_JSON. Fixed in 6f64b68 by passing shared resolved metadata; targeted CLI/contract checks passed.</t>
         </is>
       </c>
       <c r="L217" s="2" t="inlineStr">
@@ -22553,12 +22553,12 @@
       </c>
       <c r="O217" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Needs a Windows runner; failed before the CICD-01 fix and has not been rerun.</t>
+          <t xml:space="preserve">Native Windows package/EXE/WebView2 retest pending; no corrected GitHub run.</t>
         </is>
       </c>
       <c r="P217" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">docs/deployment/WINDOWS_DESKTOP.md; docs/validation/WORKFLOW_MATRIX.md</t>
+          <t xml:space="preserve">docs/deployment/WINDOWS_DESKTOP.md; docs/validation/WORKFLOW_MATRIX.md; fix: 6f64b68; docs/validation/WORKFLOW_MATRIX.md</t>
         </is>
       </c>
       <c r="Q217" s="2" t="inlineStr">
@@ -22630,7 +22630,7 @@
       </c>
       <c r="K218" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Run 41340859408 (2026-11-01): Service failed because PyInstaller resolved relative assets under the nested spec directory. Fixed in 6f64b68 with root-absolute inputs; rooted-input contract plus local PyInstaller resolver probe and PowerShell parsing passed.</t>
         </is>
       </c>
       <c r="L218" s="2" t="inlineStr">
@@ -22650,12 +22650,12 @@
       </c>
       <c r="O218" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Needs a Windows runner and a real SCM host; not run.</t>
+          <t xml:space="preserve">Windows build and SCM install/start/health/stop/uninstall still require corrected Windows job.</t>
         </is>
       </c>
       <c r="P218" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">docs/deployment/WINDOWS_SERVICE.md; docs/validation/WORKFLOW_MATRIX.md</t>
+          <t xml:space="preserve">docs/deployment/WINDOWS_SERVICE.md; docs/validation/WORKFLOW_MATRIX.md; fix: 6f64b68; docs/validation/WORKFLOW_MATRIX.md</t>
         </is>
       </c>
       <c r="Q218" s="2" t="inlineStr">
@@ -22712,7 +22712,7 @@
       </c>
       <c r="H219" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">backend/tests/test_deployment_packaging.py; backend/tests/test_deployment_contracts.py</t>
+          <t xml:space="preserve">backend/tests/test_deployment_packaging.py</t>
         </is>
       </c>
       <c r="I219" s="2" t="inlineStr">
@@ -22727,7 +22727,7 @@
       </c>
       <c r="K219" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Run 41340859408 (2026-11-01): Linux Docker packaging and verification succeeded in GitHub run 41340859408 at 513d388. Docker code unchanged by the targeted repair.</t>
         </is>
       </c>
       <c r="L219" s="2" t="inlineStr">
@@ -22747,12 +22747,12 @@
       </c>
       <c r="O219" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Docker was not run locally; no GitHub run since the change.</t>
+          <t xml:space="preserve">No new Docker job dispatched; this does not establish all target-platform acceptance.</t>
         </is>
       </c>
       <c r="P219" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">docs/deployment/LINUX_DOCKER.md; docs/validation/WORKFLOW_MATRIX.md</t>
+          <t xml:space="preserve">docs/deployment/LINUX_DOCKER.md; docs/validation/WORKFLOW_MATRIX.md; fix: 6f64b68; docs/validation/WORKFLOW_MATRIX.md</t>
         </is>
       </c>
       <c r="Q219" s="2" t="inlineStr">
@@ -22809,7 +22809,7 @@
       </c>
       <c r="H220" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">backend/tests/test_deployment_packaging.py; backend/tests/test_deployment_contracts.py</t>
+          <t xml:space="preserve">backend/tests/test_deployment_packaging.py; scripts/test-native-deployment.py</t>
         </is>
       </c>
       <c r="I220" s="2" t="inlineStr">
@@ -22824,7 +22824,7 @@
       </c>
       <c r="K220" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Run 41340859408 (2026-11-01): Native failed before vulnerability analysis: pip_audit module absent. Fixed in 6f64b68 by provisioning existing pinned audit tooling. Canonical archive, runtime audit and user-mode lifecycle passed locally.</t>
         </is>
       </c>
       <c r="L220" s="2" t="inlineStr">
@@ -22844,12 +22844,12 @@
       </c>
       <c r="O220" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Real systemd was not booted; no GitHub run since the change.</t>
+          <t xml:space="preserve">Corrected GitHub native job and real systemd acceptance pending. Wheel hashes and audit failures remain enforced.</t>
         </is>
       </c>
       <c r="P220" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">docs/deployment/LINUX_NATIVE.md; docs/validation/WORKFLOW_MATRIX.md</t>
+          <t xml:space="preserve">docs/deployment/LINUX_NATIVE.md; docs/validation/WORKFLOW_MATRIX.md; fix: 6f64b68; docs/validation/WORKFLOW_MATRIX.md</t>
         </is>
       </c>
       <c r="Q220" s="2" t="inlineStr">
@@ -23003,7 +23003,7 @@
       </c>
       <c r="H222" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">backend/tests/test_deployment_release.py; backend/tests/test_deployment_packaging.py</t>
+          <t xml:space="preserve">backend/tests/test_deployment_packaging.py; backend/tests/test_artifact_zip.py</t>
         </is>
       </c>
       <c r="I222" s="2" t="inlineStr">
@@ -23018,7 +23018,7 @@
       </c>
       <c r="K222" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Run 41340859408 (2026-11-01): Run 41340859408 native download matched expected SHA-256. digest-mismatch: error was configuration, not a detected mismatch. Integrity/receipt/provenance tests passed; controls unchanged.</t>
         </is>
       </c>
       <c r="L222" s="2" t="inlineStr">
@@ -23038,12 +23038,12 @@
       </c>
       <c r="O222" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Offline only; no real publication run.</t>
+          <t xml:space="preserve">Repaired Windows/native distribution round trips await actual GitHub jobs.</t>
         </is>
       </c>
       <c r="P222" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">docs/deployment/CI_CD.md; docs/validation/WORKFLOW_MATRIX.md</t>
+          <t xml:space="preserve">docs/deployment/CI_CD.md; docs/validation/WORKFLOW_MATRIX.md; fix: 6f64b68; docs/validation/WORKFLOW_MATRIX.md</t>
         </is>
       </c>
       <c r="Q222" s="2" t="inlineStr">
@@ -23294,7 +23294,7 @@
       </c>
       <c r="H225" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">backend/tests/test_workflows.py; backend/tests/test_deployment_packaging.py</t>
         </is>
       </c>
       <c r="I225" s="2" t="inlineStr">
@@ -23309,7 +23309,7 @@
       </c>
       <c r="K225" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Run 41340859408 (2026-11-01): Run 41340859408: selection, shared validation and Docker passed; Desktop, Service and Native failed before repairs; publish skipped. Repairs locally verified, no new workflow dispatched.</t>
         </is>
       </c>
       <c r="L225" s="2" t="inlineStr">
@@ -23329,12 +23329,12 @@
       </c>
       <c r="O225" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Fast Validation backend-only path verified (run 41335937097); the rest is pending. No workflow has been dispatched and no test release published without approval.</t>
+          <t xml:space="preserve">Minimum remaining dispatches after approval: linux-native and windows-all build-only on repaired work. Full Regression is not a prerequisite.</t>
         </is>
       </c>
       <c r="P225" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">docs/validation/WORKFLOW_MATRIX.md</t>
+          <t xml:space="preserve">docs/validation/WORKFLOW_MATRIX.md; fix: 6f64b68; docs/validation/WORKFLOW_MATRIX.md</t>
         </is>
       </c>
       <c r="Q225" s="2" t="inlineStr">

</xml_diff>